<commit_message>
Top board LCSC BOM added
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/SM_Top_PCB_DigiKey.xlsx
+++ b/Deliverables/SM_Top Board/_BOM/SM_Top_PCB_DigiKey.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B07B0D2E-E5E0-4F45-A4EE-BDC3EA2DBB92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD504608-9879-44D3-9473-36F78EB14992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -186,12 +186,6 @@
     <t>220nF</t>
   </si>
   <si>
-    <t>Cap Ceramic 0.22uF 100V X7R 10% SMD 0805 125°C Embossed T/R, CAP CER 220nF 35V 0805</t>
-  </si>
-  <si>
-    <t>08051C224K4T2A, GMK212BJ224KGHT</t>
-  </si>
-  <si>
     <t>22nF</t>
   </si>
   <si>
@@ -907,6 +901,12 @@
   </si>
   <si>
     <t>per lot has 10 pcs</t>
+  </si>
+  <si>
+    <t>Cap Ceramic 0.22uF 100V X7R 10% SMD 0805 125°C Embossed T/R</t>
+  </si>
+  <si>
+    <t>08051C224K4T2A</t>
   </si>
 </sst>
 </file>
@@ -915,7 +915,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -1028,7 +1028,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -1093,13 +1093,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1113,28 +1150,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1149,7 +1174,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="44" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1173,7 +1198,7 @@
     <xf numFmtId="44" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1191,13 +1216,34 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="2" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="5" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1502,800 +1548,800 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="31" t="s">
+        <v>206</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="32"/>
+      <c r="O1" s="32"/>
+      <c r="P1" s="32"/>
+      <c r="Q1" s="33"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="9"/>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="C2" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="F2" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="10" t="s">
+      <c r="H2" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="M2" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="N2" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="P2" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="Q2" s="7" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A3" s="9">
         <v>1</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>212</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>213</v>
-      </c>
-      <c r="I2" s="10" t="s">
-        <v>214</v>
-      </c>
-      <c r="J2" s="10" t="s">
-        <v>215</v>
-      </c>
-      <c r="K2" s="10" t="s">
-        <v>216</v>
-      </c>
-      <c r="L2" s="10" t="s">
-        <v>217</v>
-      </c>
-      <c r="M2" s="10" t="s">
-        <v>218</v>
-      </c>
-      <c r="N2" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="O2" s="11" t="s">
+      <c r="B3" s="34" t="s">
         <v>220</v>
       </c>
-      <c r="P2" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="Q2" s="10" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A3" s="12">
-        <v>1</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>222</v>
-      </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="14" t="s">
-        <v>249</v>
-      </c>
-      <c r="H3" s="26" t="s">
-        <v>273</v>
-      </c>
-      <c r="I3" s="14" t="s">
+      <c r="G3" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>271</v>
+      </c>
+      <c r="I3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="J3" s="15">
+      <c r="J3" s="11">
         <v>2</v>
       </c>
       <c r="K3" s="6">
         <f>J3*5</f>
         <v>10</v>
       </c>
-      <c r="L3" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M3" s="17">
+      <c r="L3" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M3" s="13">
         <v>1.58</v>
       </c>
-      <c r="N3" s="18">
+      <c r="N3" s="14">
         <f t="shared" ref="N3:N57" si="0">M3*J3</f>
         <v>3.16</v>
       </c>
-      <c r="O3" s="17">
+      <c r="O3" s="13">
         <v>1.2450000000000001</v>
       </c>
-      <c r="P3" s="18">
+      <c r="P3" s="14">
         <f>O3*K3</f>
         <v>12.450000000000001</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A4" s="12">
+      <c r="A4" s="9">
         <f>A3+1</f>
         <v>2</v>
       </c>
-      <c r="B4" s="13"/>
-      <c r="C4" s="14" t="s">
+      <c r="B4" s="35"/>
+      <c r="C4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="14" t="s">
-        <v>250</v>
-      </c>
-      <c r="H4" s="27" t="s">
-        <v>263</v>
-      </c>
-      <c r="I4" s="14" t="s">
+      <c r="G4" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="H4" s="23" t="s">
+        <v>261</v>
+      </c>
+      <c r="I4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="15">
+      <c r="J4" s="11">
         <v>8</v>
       </c>
       <c r="K4" s="6">
         <f t="shared" ref="K4:K57" si="1">J4*5</f>
         <v>40</v>
       </c>
-      <c r="L4" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M4" s="17">
+      <c r="L4" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M4" s="13">
         <v>0.1</v>
       </c>
-      <c r="N4" s="18">
+      <c r="N4" s="14">
         <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
-      <c r="O4" s="17">
+      <c r="O4" s="13">
         <v>4.8000000000000001E-2</v>
       </c>
-      <c r="P4" s="18">
-        <f t="shared" ref="P4:P55" si="2">O4*K4</f>
+      <c r="P4" s="14">
+        <f t="shared" ref="P4:P54" si="2">O4*K4</f>
         <v>1.92</v>
       </c>
       <c r="Q4" s="6"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="12">
-        <f t="shared" ref="A5:A57" si="3">A4+1</f>
+      <c r="A5" s="9">
+        <f t="shared" ref="A5:A56" si="3">A4+1</f>
         <v>3</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="14" t="s">
+      <c r="B5" s="35"/>
+      <c r="C5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="H5" s="27" t="s">
-        <v>264</v>
-      </c>
-      <c r="I5" s="14" t="s">
+      <c r="G5" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="H5" s="23" t="s">
+        <v>262</v>
+      </c>
+      <c r="I5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="15">
+      <c r="J5" s="11">
         <v>1</v>
       </c>
       <c r="K5" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L5" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M5" s="17">
+      <c r="L5" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M5" s="13">
         <v>0.48</v>
       </c>
-      <c r="N5" s="18">
+      <c r="N5" s="14">
         <f t="shared" si="0"/>
         <v>0.48</v>
       </c>
-      <c r="O5" s="17">
+      <c r="O5" s="13">
         <v>0.48</v>
       </c>
-      <c r="P5" s="18">
+      <c r="P5" s="14">
         <f t="shared" si="2"/>
         <v>2.4</v>
       </c>
       <c r="Q5" s="6"/>
     </row>
     <row r="6" spans="1:17" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="12">
+      <c r="A6" s="9">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="14" t="s">
+      <c r="B6" s="35"/>
+      <c r="C6" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="G6" s="14" t="s">
-        <v>252</v>
-      </c>
-      <c r="H6" s="26" t="s">
-        <v>281</v>
-      </c>
-      <c r="I6" s="14" t="s">
+      <c r="G6" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="H6" s="22" t="s">
+        <v>279</v>
+      </c>
+      <c r="I6" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="11">
         <v>1</v>
       </c>
       <c r="K6" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L6" s="16" t="s">
-        <v>282</v>
-      </c>
-      <c r="M6" s="17">
+      <c r="L6" s="12" t="s">
+        <v>280</v>
+      </c>
+      <c r="M6" s="13">
         <v>2.77</v>
       </c>
-      <c r="N6" s="18">
+      <c r="N6" s="14">
         <f>M6*J6</f>
         <v>2.77</v>
       </c>
-      <c r="O6" s="17">
+      <c r="O6" s="13">
         <v>2.77</v>
       </c>
-      <c r="P6" s="18">
+      <c r="P6" s="14">
         <f t="shared" si="2"/>
         <v>13.85</v>
       </c>
       <c r="Q6" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="12">
+      <c r="A7" s="9">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="14" t="s">
+      <c r="B7" s="35"/>
+      <c r="C7" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="14" t="s">
-        <v>249</v>
-      </c>
-      <c r="H7" s="26" t="s">
-        <v>284</v>
-      </c>
-      <c r="I7" s="14" t="s">
+      <c r="G7" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="H7" s="22" t="s">
+        <v>282</v>
+      </c>
+      <c r="I7" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="11">
         <v>1</v>
       </c>
       <c r="K7" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L7" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M7" s="17">
+      <c r="L7" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M7" s="13">
         <v>0.76</v>
       </c>
-      <c r="N7" s="18">
-        <f t="shared" ref="N7:N55" si="4">M7*J7</f>
+      <c r="N7" s="14">
+        <f t="shared" ref="N7:N54" si="4">M7*J7</f>
         <v>0.76</v>
       </c>
-      <c r="O7" s="17">
+      <c r="O7" s="13">
         <v>0.76</v>
       </c>
-      <c r="P7" s="18">
+      <c r="P7" s="14">
         <f t="shared" si="2"/>
         <v>3.8</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" s="12">
+      <c r="A8" s="9">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="B8" s="13"/>
-      <c r="C8" s="14" t="s">
+      <c r="B8" s="35"/>
+      <c r="C8" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="G8" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="H8" s="26" t="s">
-        <v>262</v>
-      </c>
-      <c r="I8" s="14" t="s">
+      <c r="G8" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="H8" s="22" t="s">
+        <v>260</v>
+      </c>
+      <c r="I8" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="J8" s="15">
+      <c r="J8" s="11">
         <v>1</v>
       </c>
       <c r="K8" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L8" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M8" s="17">
+      <c r="L8" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M8" s="13">
         <v>0.1</v>
       </c>
-      <c r="N8" s="18">
+      <c r="N8" s="14">
         <f t="shared" si="4"/>
         <v>0.1</v>
       </c>
-      <c r="O8" s="17">
+      <c r="O8" s="13">
         <v>0.1</v>
       </c>
-      <c r="P8" s="18">
+      <c r="P8" s="14">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="Q8" s="6"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="12">
+      <c r="A9" s="9">
         <f t="shared" si="3"/>
         <v>7</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="14" t="s">
+      <c r="B9" s="35"/>
+      <c r="C9" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="14" t="s">
-        <v>253</v>
-      </c>
-      <c r="H9" s="27" t="s">
-        <v>265</v>
-      </c>
-      <c r="I9" s="14" t="s">
+      <c r="G9" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="H9" s="23" t="s">
+        <v>263</v>
+      </c>
+      <c r="I9" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="J9" s="15">
+      <c r="J9" s="11">
         <v>1</v>
       </c>
       <c r="K9" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L9" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M9" s="17">
+      <c r="L9" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M9" s="13">
         <v>0.27</v>
       </c>
-      <c r="N9" s="18">
+      <c r="N9" s="14">
         <f t="shared" si="4"/>
         <v>0.27</v>
       </c>
-      <c r="O9" s="17">
+      <c r="O9" s="13">
         <v>0.27</v>
       </c>
-      <c r="P9" s="18">
+      <c r="P9" s="14">
         <f t="shared" si="2"/>
         <v>1.35</v>
       </c>
       <c r="Q9" s="6"/>
     </row>
     <row r="10" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="12">
+      <c r="A10" s="9">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="14" t="s">
+      <c r="B10" s="35"/>
+      <c r="C10" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="D10" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G10" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="H10" s="27" t="s">
-        <v>266</v>
-      </c>
-      <c r="I10" s="14" t="s">
+      <c r="G10" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>264</v>
+      </c>
+      <c r="I10" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="J10" s="15">
+      <c r="J10" s="11">
         <v>1</v>
       </c>
       <c r="K10" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L10" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M10" s="17">
+      <c r="L10" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M10" s="13">
         <v>3.1</v>
       </c>
-      <c r="N10" s="18">
+      <c r="N10" s="14">
         <f t="shared" si="4"/>
         <v>3.1</v>
       </c>
-      <c r="O10" s="17">
+      <c r="O10" s="13">
         <v>3.1</v>
       </c>
-      <c r="P10" s="18">
+      <c r="P10" s="14">
         <f t="shared" si="2"/>
         <v>15.5</v>
       </c>
       <c r="Q10" s="6" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="12">
+      <c r="A11" s="9">
         <f t="shared" si="3"/>
         <v>9</v>
       </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="14" t="s">
+      <c r="B11" s="35"/>
+      <c r="C11" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="G11" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="H11" s="26" t="s">
-        <v>262</v>
-      </c>
-      <c r="I11" s="14" t="s">
+      <c r="G11" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="H11" s="22" t="s">
+        <v>260</v>
+      </c>
+      <c r="I11" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J11" s="15">
+      <c r="J11" s="11">
         <v>1</v>
       </c>
       <c r="K11" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L11" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M11" s="17">
+      <c r="L11" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M11" s="13">
         <v>0.12</v>
       </c>
-      <c r="N11" s="18">
+      <c r="N11" s="14">
         <f t="shared" si="4"/>
         <v>0.12</v>
       </c>
-      <c r="O11" s="17">
+      <c r="O11" s="13">
         <v>0.12</v>
       </c>
-      <c r="P11" s="18">
+      <c r="P11" s="14">
         <f t="shared" si="2"/>
         <v>0.6</v>
       </c>
       <c r="Q11" s="6"/>
     </row>
     <row r="12" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="12">
+      <c r="A12" s="9">
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="14" t="s">
+      <c r="B12" s="35"/>
+      <c r="C12" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="G12" s="14" t="s">
-        <v>254</v>
-      </c>
-      <c r="H12" s="27" t="s">
-        <v>267</v>
-      </c>
-      <c r="I12" s="14" t="s">
+      <c r="G12" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="H12" s="23" t="s">
+        <v>265</v>
+      </c>
+      <c r="I12" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="J12" s="15">
+      <c r="J12" s="11">
         <v>5</v>
       </c>
       <c r="K12" s="6">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="L12" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M12" s="17">
+      <c r="L12" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M12" s="13">
         <v>0.21</v>
       </c>
-      <c r="N12" s="18">
+      <c r="N12" s="14">
         <f t="shared" si="4"/>
         <v>1.05</v>
       </c>
-      <c r="O12" s="17">
+      <c r="O12" s="13">
         <v>0.14299999999999999</v>
       </c>
-      <c r="P12" s="18">
+      <c r="P12" s="14">
         <f t="shared" si="2"/>
         <v>3.5749999999999997</v>
       </c>
       <c r="Q12" s="6"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" s="12">
+      <c r="A13" s="9">
         <f t="shared" si="3"/>
         <v>11</v>
       </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="14" t="s">
+      <c r="B13" s="35"/>
+      <c r="C13" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="G13" s="14" t="s">
-        <v>250</v>
-      </c>
-      <c r="H13" s="27" t="s">
-        <v>268</v>
-      </c>
-      <c r="I13" s="14" t="s">
+      <c r="G13" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="H13" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="I13" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="J13" s="15">
+      <c r="J13" s="11">
         <v>2</v>
       </c>
       <c r="K13" s="6">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L13" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M13" s="17">
+      <c r="L13" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M13" s="13">
         <v>0.31</v>
       </c>
-      <c r="N13" s="18">
+      <c r="N13" s="14">
         <f t="shared" si="4"/>
         <v>0.62</v>
       </c>
-      <c r="O13" s="17">
+      <c r="O13" s="13">
         <v>0.14299999999999999</v>
       </c>
-      <c r="P13" s="18">
+      <c r="P13" s="14">
         <f t="shared" si="2"/>
         <v>1.43</v>
       </c>
       <c r="Q13" s="6"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A14" s="12">
+      <c r="A14" s="9">
         <f t="shared" si="3"/>
         <v>12</v>
       </c>
-      <c r="B14" s="13"/>
-      <c r="C14" s="14" t="s">
+      <c r="B14" s="35"/>
+      <c r="C14" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="14" t="s">
+      <c r="E14" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="G14" s="14" t="s">
-        <v>250</v>
-      </c>
-      <c r="H14" s="28" t="s">
-        <v>269</v>
-      </c>
-      <c r="I14" s="14" t="s">
+      <c r="G14" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="H14" s="24" t="s">
+        <v>267</v>
+      </c>
+      <c r="I14" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="J14" s="15">
+      <c r="J14" s="11">
         <v>2</v>
       </c>
       <c r="K14" s="6">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L14" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M14" s="17">
+      <c r="L14" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M14" s="13">
         <v>0.19</v>
       </c>
-      <c r="N14" s="18">
+      <c r="N14" s="14">
         <f t="shared" si="4"/>
         <v>0.38</v>
       </c>
-      <c r="O14" s="17">
+      <c r="O14" s="13">
         <v>0.13500000000000001</v>
       </c>
-      <c r="P14" s="18">
+      <c r="P14" s="14">
         <f t="shared" si="2"/>
         <v>1.35</v>
       </c>
       <c r="Q14" s="6"/>
     </row>
     <row r="15" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="12">
+      <c r="A15" s="9">
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="D15" s="14" t="s">
-        <v>289</v>
-      </c>
-      <c r="E15" s="14" t="s">
+      <c r="B15" s="35"/>
+      <c r="C15" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="F15" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="G15" s="14" t="s">
-        <v>255</v>
-      </c>
-      <c r="H15" s="26" t="s">
-        <v>262</v>
-      </c>
-      <c r="I15" s="14" t="s">
+      <c r="F15" s="10" t="s">
+        <v>293</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="H15" s="22" t="s">
+        <v>260</v>
+      </c>
+      <c r="I15" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="J15" s="15">
+      <c r="J15" s="11">
         <v>4</v>
       </c>
       <c r="K15" s="6">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L15" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M15" s="17">
+      <c r="L15" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M15" s="13">
         <v>0.27</v>
       </c>
-      <c r="N15" s="18">
+      <c r="N15" s="14">
         <f t="shared" si="4"/>
         <v>1.08</v>
       </c>
-      <c r="O15" s="17">
+      <c r="O15" s="13">
         <v>0.185</v>
       </c>
-      <c r="P15" s="18">
+      <c r="P15" s="14">
         <f t="shared" si="2"/>
         <v>3.7</v>
       </c>
-      <c r="Q15" s="19"/>
+      <c r="Q15" s="15"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A16" s="12">
+      <c r="A16" s="9">
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="B16" s="13"/>
+      <c r="B16" s="35"/>
       <c r="C16" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="E16" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>288</v>
-      </c>
       <c r="G16" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="H16" s="29" t="s">
-        <v>262</v>
+        <v>251</v>
+      </c>
+      <c r="H16" s="25" t="s">
+        <v>260</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>52</v>
@@ -2308,213 +2354,213 @@
         <v>20</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="M16" s="5">
         <v>0.21</v>
       </c>
-      <c r="N16" s="18">
+      <c r="N16" s="14">
         <f t="shared" si="4"/>
         <v>0.84</v>
       </c>
       <c r="O16" s="5">
         <v>0.14899999999999999</v>
       </c>
-      <c r="P16" s="18">
+      <c r="P16" s="14">
         <f t="shared" si="2"/>
         <v>2.98</v>
       </c>
       <c r="Q16" s="6"/>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A17" s="12">
+      <c r="A17" s="9">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="14" t="s">
+      <c r="B17" s="35"/>
+      <c r="C17" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="D17" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="F17" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="G17" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="H17" s="26" t="s">
-        <v>262</v>
-      </c>
-      <c r="I17" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="J17" s="15">
+      <c r="G17" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="H17" s="22" t="s">
+        <v>260</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="J17" s="11">
         <v>1</v>
       </c>
       <c r="K17" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L17" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M17" s="17">
+      <c r="L17" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M17" s="13">
         <v>0.11</v>
       </c>
-      <c r="N17" s="18">
+      <c r="N17" s="14">
         <f t="shared" si="4"/>
         <v>0.11</v>
       </c>
-      <c r="O17" s="17">
+      <c r="O17" s="13">
         <v>0.11</v>
       </c>
-      <c r="P17" s="18">
+      <c r="P17" s="14">
         <f t="shared" si="2"/>
         <v>0.55000000000000004</v>
       </c>
       <c r="Q17" s="6"/>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A18" s="12">
+      <c r="A18" s="9">
         <f t="shared" si="3"/>
         <v>16</v>
       </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="14" t="s">
+      <c r="B18" s="35"/>
+      <c r="C18" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="E18" s="14" t="s">
+      <c r="D18" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E18" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="F18" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="G18" s="14" t="s">
-        <v>253</v>
-      </c>
-      <c r="H18" s="26" t="s">
-        <v>262</v>
-      </c>
-      <c r="I18" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="J18" s="15">
+      <c r="G18" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="H18" s="22" t="s">
+        <v>260</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="J18" s="11">
         <v>1</v>
       </c>
       <c r="K18" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L18" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M18" s="17">
+      <c r="L18" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M18" s="13">
         <v>0.21</v>
       </c>
-      <c r="N18" s="18">
+      <c r="N18" s="14">
         <f t="shared" si="4"/>
         <v>0.21</v>
       </c>
-      <c r="O18" s="17">
+      <c r="O18" s="13">
         <v>0.14899999999999999</v>
       </c>
-      <c r="P18" s="18">
+      <c r="P18" s="14">
         <f t="shared" si="2"/>
         <v>0.745</v>
       </c>
-      <c r="Q18" s="19"/>
+      <c r="Q18" s="15"/>
     </row>
     <row r="19" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="12">
+      <c r="A19" s="9">
         <f t="shared" si="3"/>
         <v>17</v>
       </c>
-      <c r="B19" s="13" t="s">
-        <v>223</v>
-      </c>
-      <c r="C19" s="14" t="s">
+      <c r="B19" s="36"/>
+      <c r="C19" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E19" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="F19" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="E19" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F19" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="G19" s="14" t="s">
-        <v>253</v>
-      </c>
-      <c r="H19" s="28" t="s">
-        <v>265</v>
-      </c>
-      <c r="I19" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="J19" s="15">
+      <c r="G19" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>263</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="J19" s="11">
         <v>4</v>
       </c>
       <c r="K19" s="6">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L19" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M19" s="17">
+      <c r="L19" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M19" s="13">
         <v>0.27</v>
       </c>
-      <c r="N19" s="18">
+      <c r="N19" s="14">
         <f t="shared" si="4"/>
         <v>1.08</v>
       </c>
-      <c r="O19" s="17">
+      <c r="O19" s="13">
         <v>0.27</v>
       </c>
-      <c r="P19" s="18">
+      <c r="P19" s="14">
         <f t="shared" si="2"/>
         <v>5.4</v>
       </c>
       <c r="Q19" s="6"/>
     </row>
     <row r="20" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="12">
+      <c r="A20" s="9">
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="B20" s="13"/>
-      <c r="C20" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="E20" s="14" t="s">
+      <c r="B20" s="34" t="s">
+        <v>221</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="F20" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>250</v>
-      </c>
-      <c r="H20" s="28" t="s">
-        <v>270</v>
-      </c>
-      <c r="I20" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="J20" s="15">
+      <c r="E20" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="H20" s="24" t="s">
+        <v>268</v>
+      </c>
+      <c r="I20" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="J20" s="11">
         <v>1</v>
       </c>
       <c r="K20" s="6">
@@ -2522,54 +2568,54 @@
         <v>5</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="M20" s="5">
         <v>0.75</v>
       </c>
-      <c r="N20" s="18">
+      <c r="N20" s="14">
         <f t="shared" si="4"/>
         <v>0.75</v>
       </c>
       <c r="O20" s="5">
         <v>0.75</v>
       </c>
-      <c r="P20" s="18">
+      <c r="P20" s="14">
         <f t="shared" si="2"/>
         <v>3.75</v>
       </c>
-      <c r="Q20" s="19" t="s">
-        <v>248</v>
+      <c r="Q20" s="15" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="21" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="12">
+      <c r="A21" s="9">
         <f t="shared" si="3"/>
         <v>19</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="14" t="s">
+      <c r="B21" s="35"/>
+      <c r="C21" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="E21" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="D21" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="F21" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="G21" s="14" t="s">
-        <v>256</v>
-      </c>
-      <c r="H21" s="28" t="s">
-        <v>271</v>
-      </c>
-      <c r="I21" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="J21" s="15">
+      <c r="F21" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>254</v>
+      </c>
+      <c r="H21" s="24" t="s">
+        <v>269</v>
+      </c>
+      <c r="I21" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="J21" s="11">
         <v>8</v>
       </c>
       <c r="K21" s="6">
@@ -2577,109 +2623,107 @@
         <v>40</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="M21" s="5">
         <v>0.42</v>
       </c>
-      <c r="N21" s="18">
+      <c r="N21" s="14">
         <f t="shared" si="4"/>
         <v>3.36</v>
       </c>
       <c r="O21" s="5">
         <v>0.313</v>
       </c>
-      <c r="P21" s="18">
+      <c r="P21" s="14">
         <f t="shared" si="2"/>
         <v>12.52</v>
       </c>
-      <c r="Q21" s="19" t="s">
-        <v>248</v>
+      <c r="Q21" s="15" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A22" s="12">
+      <c r="A22" s="9">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="B22" s="13"/>
-      <c r="C22" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="E22" s="14" t="s">
+      <c r="B22" s="35"/>
+      <c r="C22" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="D22" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="F22" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="G22" s="14" t="s">
-        <v>257</v>
-      </c>
-      <c r="H22" s="28" t="s">
-        <v>290</v>
-      </c>
-      <c r="I22" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="J22" s="15">
+      <c r="E22" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="G22" s="10" t="s">
+        <v>255</v>
+      </c>
+      <c r="H22" s="24" t="s">
+        <v>288</v>
+      </c>
+      <c r="I22" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="J22" s="11">
         <v>1</v>
       </c>
       <c r="K22" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L22" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M22" s="17">
+      <c r="L22" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M22" s="13">
         <v>0.5</v>
       </c>
-      <c r="N22" s="18">
+      <c r="N22" s="14">
         <f t="shared" si="4"/>
         <v>0.5</v>
       </c>
-      <c r="O22" s="17">
+      <c r="O22" s="13">
         <v>0.5</v>
       </c>
-      <c r="P22" s="18">
+      <c r="P22" s="14">
         <f t="shared" si="2"/>
         <v>2.5</v>
       </c>
       <c r="Q22" s="6"/>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A23" s="12">
+      <c r="A23" s="9">
         <f t="shared" si="3"/>
         <v>21</v>
       </c>
-      <c r="B23" s="12" t="s">
-        <v>224</v>
-      </c>
-      <c r="C23" s="14" t="s">
+      <c r="B23" s="36"/>
+      <c r="C23" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="E23" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="D23" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="E23" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="F23" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="G23" s="14" t="s">
-        <v>258</v>
-      </c>
-      <c r="H23" s="14" t="s">
-        <v>262</v>
-      </c>
-      <c r="I23" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="J23" s="15">
+      <c r="F23" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="G23" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="H23" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="I23" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="J23" s="11">
         <v>1</v>
       </c>
       <c r="K23" s="6">
@@ -2687,54 +2731,54 @@
         <v>5</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="M23" s="5">
         <v>0.37</v>
       </c>
-      <c r="N23" s="18">
+      <c r="N23" s="14">
         <f t="shared" si="4"/>
         <v>0.37</v>
       </c>
       <c r="O23" s="5">
         <v>0.37</v>
       </c>
-      <c r="P23" s="18">
+      <c r="P23" s="14">
         <f t="shared" si="2"/>
         <v>1.85</v>
       </c>
-      <c r="Q23" s="19"/>
+      <c r="Q23" s="15"/>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A24" s="12">
+      <c r="A24" s="9">
         <f t="shared" si="3"/>
         <v>22</v>
       </c>
-      <c r="B24" s="12" t="s">
-        <v>226</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="D24" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E24" s="14" t="s">
+      <c r="B24" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="D24" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="F24" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="G24" s="14" t="s">
-        <v>259</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>262</v>
-      </c>
-      <c r="I24" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="J24" s="15">
+      <c r="E24" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="G24" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="I24" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="J24" s="11">
         <v>1</v>
       </c>
       <c r="K24" s="6">
@@ -2743,47 +2787,47 @@
       </c>
       <c r="L24" s="1"/>
       <c r="M24" s="5"/>
-      <c r="N24" s="18">
+      <c r="N24" s="14">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="O24" s="5"/>
-      <c r="P24" s="18">
+      <c r="P24" s="14">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Q24" s="6"/>
     </row>
     <row r="25" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="12">
+      <c r="A25" s="9">
         <f t="shared" si="3"/>
         <v>23</v>
       </c>
-      <c r="B25" s="12" t="s">
-        <v>225</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="D25" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="E25" s="14" t="s">
+      <c r="B25" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="D25" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="F25" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="G25" s="14" t="s">
+      <c r="E25" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="H25" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="H25" s="14" t="s">
-        <v>262</v>
-      </c>
-      <c r="I25" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="J25" s="15">
+      <c r="I25" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J25" s="11">
         <v>1</v>
       </c>
       <c r="K25" s="6">
@@ -2791,54 +2835,54 @@
         <v>5</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="M25" s="5">
         <v>2.75</v>
       </c>
-      <c r="N25" s="18">
+      <c r="N25" s="14">
         <f t="shared" si="4"/>
         <v>2.75</v>
       </c>
       <c r="O25" s="5">
         <v>2.75</v>
       </c>
-      <c r="P25" s="18">
+      <c r="P25" s="14">
         <f t="shared" si="2"/>
         <v>13.75</v>
       </c>
       <c r="Q25" s="6"/>
     </row>
     <row r="26" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A26" s="12">
+      <c r="A26" s="9">
         <f t="shared" si="3"/>
         <v>24</v>
       </c>
-      <c r="B26" s="13" t="s">
-        <v>227</v>
-      </c>
-      <c r="C26" s="14" t="s">
+      <c r="B26" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="E26" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="D26" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="E26" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="F26" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="G26" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="H26" s="14" t="s">
-        <v>262</v>
-      </c>
-      <c r="I26" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="J26" s="15">
+      <c r="F26" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="G26" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="H26" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="I26" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="J26" s="11">
         <v>8</v>
       </c>
       <c r="K26" s="6">
@@ -2846,52 +2890,54 @@
         <v>40</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="M26" s="5">
         <v>1.92</v>
       </c>
-      <c r="N26" s="18">
+      <c r="N26" s="14">
         <f t="shared" si="4"/>
         <v>15.36</v>
       </c>
       <c r="O26" s="5">
         <v>1.6332</v>
       </c>
-      <c r="P26" s="18">
+      <c r="P26" s="14">
         <f t="shared" si="2"/>
         <v>65.328000000000003</v>
       </c>
       <c r="Q26" s="6"/>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A27" s="12">
+      <c r="A27" s="9">
         <f t="shared" si="3"/>
         <v>25</v>
       </c>
-      <c r="B27" s="13"/>
-      <c r="C27" s="14" t="s">
+      <c r="B27" s="34" t="s">
+        <v>225</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F27" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="D27" s="14" t="s">
-        <v>116</v>
-      </c>
-      <c r="E27" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F27" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="G27" s="14" t="s">
-        <v>261</v>
-      </c>
-      <c r="H27" s="14" t="s">
-        <v>262</v>
-      </c>
-      <c r="I27" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="J27" s="15">
+      <c r="G27" s="10" t="s">
+        <v>259</v>
+      </c>
+      <c r="H27" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="I27" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="J27" s="11">
         <v>2</v>
       </c>
       <c r="K27" s="6">
@@ -2899,52 +2945,52 @@
         <v>10</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="M27" s="5">
         <v>0.1</v>
       </c>
-      <c r="N27" s="18">
+      <c r="N27" s="14">
         <f t="shared" si="4"/>
         <v>0.2</v>
       </c>
       <c r="O27" s="5">
         <v>0.02</v>
       </c>
-      <c r="P27" s="18">
+      <c r="P27" s="14">
         <f t="shared" si="2"/>
         <v>0.2</v>
       </c>
       <c r="Q27" s="6"/>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A28" s="12">
+      <c r="A28" s="9">
         <f t="shared" si="3"/>
         <v>26</v>
       </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="14" t="s">
+      <c r="B28" s="35"/>
+      <c r="C28" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F28" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="D28" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="E28" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F28" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="G28" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="H28" s="14" t="s">
-        <v>262</v>
-      </c>
-      <c r="I28" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="J28" s="15">
+      <c r="G28" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="H28" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="I28" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="J28" s="11">
         <v>2</v>
       </c>
       <c r="K28" s="6">
@@ -2952,52 +2998,52 @@
         <v>10</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="M28" s="5">
         <v>0.1</v>
       </c>
-      <c r="N28" s="18">
+      <c r="N28" s="14">
         <f t="shared" si="4"/>
         <v>0.2</v>
       </c>
       <c r="O28" s="5">
         <v>1.7999999999999999E-2</v>
       </c>
-      <c r="P28" s="18">
+      <c r="P28" s="14">
         <f t="shared" si="2"/>
         <v>0.18</v>
       </c>
       <c r="Q28" s="6"/>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A29" s="12">
+      <c r="A29" s="9">
         <f t="shared" si="3"/>
         <v>27</v>
       </c>
-      <c r="B29" s="13"/>
-      <c r="C29" s="14" t="s">
+      <c r="B29" s="35"/>
+      <c r="C29" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F29" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="D29" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="E29" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F29" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="G29" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="H29" s="14" t="s">
-        <v>262</v>
-      </c>
-      <c r="I29" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="J29" s="15">
+      <c r="G29" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="H29" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="I29" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="J29" s="11">
         <v>1</v>
       </c>
       <c r="K29" s="6">
@@ -3005,1461 +3051,1461 @@
         <v>5</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="M29" s="5">
         <v>0.1</v>
       </c>
-      <c r="N29" s="18">
+      <c r="N29" s="14">
         <f t="shared" si="4"/>
         <v>0.1</v>
       </c>
       <c r="O29" s="5">
         <v>0.1</v>
       </c>
-      <c r="P29" s="18">
+      <c r="P29" s="14">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="Q29" s="6"/>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A30" s="12">
+      <c r="A30" s="9">
         <f t="shared" si="3"/>
         <v>28</v>
       </c>
-      <c r="B30" s="13"/>
-      <c r="C30" s="14" t="s">
+      <c r="B30" s="35"/>
+      <c r="C30" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F30" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="D30" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="E30" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F30" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="G30" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="H30" s="14" t="s">
-        <v>262</v>
-      </c>
-      <c r="I30" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J30" s="15">
+      <c r="G30" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="H30" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="I30" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="J30" s="11">
         <v>1</v>
       </c>
       <c r="K30" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L30" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="M30" s="17">
+      <c r="L30" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="M30" s="13">
         <v>0.1</v>
       </c>
-      <c r="N30" s="18">
+      <c r="N30" s="14">
         <f t="shared" si="4"/>
         <v>0.1</v>
       </c>
-      <c r="O30" s="17">
+      <c r="O30" s="13">
         <v>0.1</v>
       </c>
-      <c r="P30" s="18">
+      <c r="P30" s="14">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="Q30" s="6"/>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A31" s="12">
+      <c r="A31" s="9">
         <f t="shared" si="3"/>
         <v>29</v>
       </c>
-      <c r="B31" s="13"/>
-      <c r="C31" s="14" t="s">
+      <c r="B31" s="35"/>
+      <c r="C31" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F31" s="10" t="s">
         <v>131</v>
-      </c>
-      <c r="D31" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="E31" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F31" s="14" t="s">
-        <v>133</v>
       </c>
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
-      <c r="I31" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="J31" s="15">
+      <c r="I31" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="J31" s="11">
         <v>4</v>
       </c>
       <c r="K31" s="6">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L31" s="21" t="s">
-        <v>233</v>
-      </c>
-      <c r="M31" s="17">
+      <c r="L31" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="M31" s="13">
         <v>0.1</v>
       </c>
-      <c r="N31" s="18">
+      <c r="N31" s="14">
         <f t="shared" si="4"/>
         <v>0.4</v>
       </c>
-      <c r="O31" s="17">
+      <c r="O31" s="13">
         <v>2.4E-2</v>
       </c>
-      <c r="P31" s="18">
+      <c r="P31" s="14">
         <f t="shared" si="2"/>
         <v>0.48</v>
       </c>
       <c r="Q31" s="6"/>
     </row>
     <row r="32" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A32" s="12">
+      <c r="A32" s="9">
         <f t="shared" si="3"/>
         <v>30</v>
       </c>
-      <c r="B32" s="13"/>
-      <c r="C32" s="14" t="s">
+      <c r="B32" s="35"/>
+      <c r="C32" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D32" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="E32" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D32" s="14" t="s">
+      <c r="F32" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="E32" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="F32" s="14" t="s">
-        <v>138</v>
-      </c>
       <c r="G32" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="I32" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="J32" s="11">
+        <v>4</v>
+      </c>
+      <c r="K32" s="6">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="L32" s="12" t="s">
         <v>231</v>
       </c>
-      <c r="H32" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="I32" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="J32" s="15">
-        <v>4</v>
-      </c>
-      <c r="K32" s="6">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-      <c r="L32" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M32" s="17">
+      <c r="M32" s="13">
         <v>1.28</v>
       </c>
-      <c r="N32" s="18">
+      <c r="N32" s="14">
         <f t="shared" si="4"/>
         <v>5.12</v>
       </c>
-      <c r="O32" s="17">
+      <c r="O32" s="13">
         <v>1.135</v>
       </c>
-      <c r="P32" s="18">
+      <c r="P32" s="14">
         <f t="shared" si="2"/>
         <v>22.7</v>
       </c>
       <c r="Q32" s="6"/>
     </row>
     <row r="33" spans="1:17" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A33" s="12">
+      <c r="A33" s="9">
         <f t="shared" si="3"/>
         <v>31</v>
       </c>
-      <c r="B33" s="13"/>
-      <c r="C33" s="14" t="s">
+      <c r="B33" s="35"/>
+      <c r="C33" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F33" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="D33" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="E33" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F33" s="14" t="s">
-        <v>142</v>
-      </c>
       <c r="G33" s="6" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H33" s="6"/>
-      <c r="I33" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="J33" s="15">
+      <c r="I33" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="J33" s="11">
         <v>8</v>
       </c>
       <c r="K33" s="6">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="L33" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M33" s="17">
+      <c r="L33" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M33" s="13">
         <v>0.1</v>
       </c>
-      <c r="N33" s="18">
+      <c r="N33" s="14">
         <f t="shared" si="4"/>
         <v>0.8</v>
       </c>
-      <c r="O33" s="17">
+      <c r="O33" s="13">
         <v>2.4E-2</v>
       </c>
-      <c r="P33" s="18">
+      <c r="P33" s="14">
         <f t="shared" si="2"/>
         <v>0.96</v>
       </c>
       <c r="Q33" s="6"/>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A34" s="12">
+      <c r="A34" s="9">
         <f t="shared" si="3"/>
         <v>32</v>
       </c>
-      <c r="B34" s="13"/>
-      <c r="C34" s="14" t="s">
+      <c r="B34" s="35"/>
+      <c r="C34" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F34" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="D34" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="E34" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F34" s="14" t="s">
-        <v>146</v>
-      </c>
       <c r="G34" s="6" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>236</v>
-      </c>
-      <c r="I34" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="J34" s="15">
+        <v>234</v>
+      </c>
+      <c r="I34" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="J34" s="11">
         <v>1</v>
       </c>
       <c r="K34" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L34" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M34" s="17">
+      <c r="L34" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M34" s="13">
         <v>0.1</v>
       </c>
-      <c r="N34" s="18">
+      <c r="N34" s="14">
         <f t="shared" si="4"/>
         <v>0.1</v>
       </c>
-      <c r="O34" s="17">
+      <c r="O34" s="13">
         <v>0.1</v>
       </c>
-      <c r="P34" s="18">
+      <c r="P34" s="14">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="Q34" s="6"/>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A35" s="12">
+      <c r="A35" s="9">
         <f t="shared" si="3"/>
         <v>33</v>
       </c>
-      <c r="B35" s="13"/>
-      <c r="C35" s="14" t="s">
+      <c r="B35" s="35"/>
+      <c r="C35" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F35" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="D35" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="E35" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F35" s="14" t="s">
-        <v>150</v>
-      </c>
       <c r="G35" s="6" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H35" s="6"/>
-      <c r="I35" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="J35" s="15">
+      <c r="I35" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="J35" s="11">
         <v>1</v>
       </c>
       <c r="K35" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L35" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M35" s="17">
+      <c r="L35" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M35" s="13">
         <v>0.1</v>
       </c>
-      <c r="N35" s="18">
+      <c r="N35" s="14">
         <f t="shared" si="4"/>
         <v>0.1</v>
       </c>
-      <c r="O35" s="17">
+      <c r="O35" s="13">
         <v>0.1</v>
       </c>
-      <c r="P35" s="18">
+      <c r="P35" s="14">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="Q35" s="6"/>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A36" s="12">
+      <c r="A36" s="9">
         <f t="shared" si="3"/>
         <v>34</v>
       </c>
-      <c r="B36" s="13"/>
-      <c r="C36" s="14" t="s">
+      <c r="B36" s="35"/>
+      <c r="C36" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F36" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="D36" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="E36" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F36" s="14" t="s">
-        <v>154</v>
-      </c>
       <c r="G36" s="6" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H36" s="6"/>
-      <c r="I36" s="14" t="s">
-        <v>151</v>
-      </c>
-      <c r="J36" s="15">
+      <c r="I36" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="J36" s="11">
         <v>1</v>
       </c>
       <c r="K36" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L36" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M36" s="17">
+      <c r="L36" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M36" s="13">
         <v>0.1</v>
       </c>
-      <c r="N36" s="18">
+      <c r="N36" s="14">
         <f t="shared" si="4"/>
         <v>0.1</v>
       </c>
-      <c r="O36" s="17">
+      <c r="O36" s="13">
         <v>0.1</v>
       </c>
-      <c r="P36" s="18">
+      <c r="P36" s="14">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="Q36" s="6"/>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A37" s="12">
+      <c r="A37" s="9">
         <f t="shared" si="3"/>
         <v>35</v>
       </c>
-      <c r="B37" s="13"/>
-      <c r="C37" s="14" t="s">
+      <c r="B37" s="35"/>
+      <c r="C37" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F37" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="D37" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="E37" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F37" s="14" t="s">
-        <v>158</v>
-      </c>
       <c r="G37" s="6" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H37" s="6"/>
-      <c r="I37" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="J37" s="15">
+      <c r="I37" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="J37" s="11">
         <v>1</v>
       </c>
       <c r="K37" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L37" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M37" s="17">
+      <c r="L37" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M37" s="13">
         <v>0.1</v>
       </c>
-      <c r="N37" s="18">
+      <c r="N37" s="14">
         <f t="shared" si="4"/>
         <v>0.1</v>
       </c>
-      <c r="O37" s="17">
+      <c r="O37" s="13">
         <v>0.1</v>
       </c>
-      <c r="P37" s="18">
+      <c r="P37" s="14">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="Q37" s="6"/>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A38" s="12">
+      <c r="A38" s="9">
         <f t="shared" si="3"/>
         <v>36</v>
       </c>
-      <c r="B38" s="13"/>
-      <c r="C38" s="14" t="s">
+      <c r="B38" s="35"/>
+      <c r="C38" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F38" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="D38" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="E38" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F38" s="14" t="s">
-        <v>162</v>
-      </c>
       <c r="G38" s="6" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H38" s="6"/>
-      <c r="I38" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="J38" s="15">
+      <c r="I38" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="J38" s="11">
         <v>1</v>
       </c>
       <c r="K38" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L38" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M38" s="17">
+      <c r="L38" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M38" s="13">
         <v>0.1</v>
       </c>
-      <c r="N38" s="18">
+      <c r="N38" s="14">
         <f t="shared" si="4"/>
         <v>0.1</v>
       </c>
-      <c r="O38" s="17">
+      <c r="O38" s="13">
         <v>0.1</v>
       </c>
-      <c r="P38" s="18">
+      <c r="P38" s="14">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="Q38" s="6"/>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A39" s="12">
+      <c r="A39" s="9">
         <f t="shared" si="3"/>
         <v>37</v>
       </c>
-      <c r="B39" s="13"/>
-      <c r="C39" s="14" t="s">
+      <c r="B39" s="35"/>
+      <c r="C39" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F39" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="D39" s="14" t="s">
-        <v>165</v>
-      </c>
-      <c r="E39" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F39" s="14" t="s">
-        <v>166</v>
-      </c>
       <c r="G39" s="6" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="I39" s="14" t="s">
-        <v>163</v>
-      </c>
-      <c r="J39" s="15">
+        <v>235</v>
+      </c>
+      <c r="I39" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="J39" s="11">
         <v>1</v>
       </c>
       <c r="K39" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L39" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M39" s="17">
+      <c r="L39" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M39" s="13">
         <v>0.38</v>
       </c>
-      <c r="N39" s="18">
+      <c r="N39" s="14">
         <f t="shared" si="4"/>
         <v>0.38</v>
       </c>
-      <c r="O39" s="17">
+      <c r="O39" s="13">
         <v>0.38</v>
       </c>
-      <c r="P39" s="18">
+      <c r="P39" s="14">
         <f t="shared" si="2"/>
         <v>1.9</v>
       </c>
       <c r="Q39" s="6"/>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A40" s="12">
+      <c r="A40" s="9">
         <f t="shared" si="3"/>
         <v>38</v>
       </c>
-      <c r="B40" s="13" t="s">
-        <v>228</v>
-      </c>
-      <c r="C40" s="14" t="s">
+      <c r="B40" s="36"/>
+      <c r="C40" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F40" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="D40" s="14" t="s">
-        <v>169</v>
-      </c>
-      <c r="E40" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F40" s="14" t="s">
-        <v>170</v>
-      </c>
       <c r="G40" s="6" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H40" s="6"/>
-      <c r="I40" s="14" t="s">
-        <v>167</v>
-      </c>
-      <c r="J40" s="15">
+      <c r="I40" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="J40" s="11">
         <v>1</v>
       </c>
       <c r="K40" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L40" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M40" s="17">
+      <c r="L40" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M40" s="13">
         <v>0.1</v>
       </c>
-      <c r="N40" s="18">
+      <c r="N40" s="14">
         <f t="shared" si="4"/>
         <v>0.1</v>
       </c>
-      <c r="O40" s="17">
+      <c r="O40" s="13">
         <v>0.1</v>
       </c>
-      <c r="P40" s="18">
+      <c r="P40" s="14">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="Q40" s="6"/>
     </row>
     <row r="41" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A41" s="12">
+      <c r="A41" s="9">
         <f t="shared" si="3"/>
         <v>39</v>
       </c>
-      <c r="B41" s="13"/>
-      <c r="C41" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="D41" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="E41" s="14" t="s">
+      <c r="B41" s="34" t="s">
+        <v>226</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="D41" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="F41" s="14" t="s">
-        <v>174</v>
+      <c r="E41" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="F41" s="10" t="s">
+        <v>172</v>
       </c>
       <c r="G41" s="6"/>
       <c r="H41" s="6"/>
-      <c r="I41" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="J41" s="15">
+      <c r="I41" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="J41" s="11">
         <v>1</v>
       </c>
       <c r="K41" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L41" s="16" t="s">
-        <v>238</v>
-      </c>
-      <c r="M41" s="17">
+      <c r="L41" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="M41" s="13">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="N41" s="18">
+      <c r="N41" s="14">
         <f t="shared" si="4"/>
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="O41" s="17">
+      <c r="O41" s="13">
         <v>1.8</v>
       </c>
-      <c r="P41" s="18">
+      <c r="P41" s="14">
         <v>1.8</v>
       </c>
       <c r="Q41" s="6" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="42" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A42" s="12">
+      <c r="A42" s="9">
         <f t="shared" si="3"/>
         <v>40</v>
       </c>
-      <c r="B42" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="C42" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="D42" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="E42" s="14" t="s">
+      <c r="B42" s="36"/>
+      <c r="C42" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="D42" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="F42" s="14" t="s">
-        <v>177</v>
+      <c r="E42" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="F42" s="10" t="s">
+        <v>175</v>
       </c>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
-      <c r="I42" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="J42" s="15">
+      <c r="I42" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="J42" s="11">
         <v>2</v>
       </c>
       <c r="K42" s="6">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L42" s="21" t="s">
-        <v>280</v>
-      </c>
-      <c r="M42" s="17">
+      <c r="L42" s="17" t="s">
+        <v>278</v>
+      </c>
+      <c r="M42" s="13">
         <v>0.34</v>
       </c>
-      <c r="N42" s="18">
+      <c r="N42" s="14">
         <f t="shared" si="4"/>
         <v>0.68</v>
       </c>
-      <c r="O42" s="17">
+      <c r="O42" s="13">
         <v>0.26</v>
       </c>
-      <c r="P42" s="18">
+      <c r="P42" s="14">
         <f t="shared" si="2"/>
         <v>2.6</v>
       </c>
       <c r="Q42" s="6"/>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A43" s="12">
+      <c r="A43" s="9">
         <f t="shared" si="3"/>
         <v>41</v>
       </c>
-      <c r="B43" s="13"/>
-      <c r="C43" s="14" t="s">
+      <c r="B43" s="34" t="s">
+        <v>227</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="E43" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="D43" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="E43" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="F43" s="14" t="s">
-        <v>180</v>
+      <c r="F43" s="10" t="s">
+        <v>178</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H43" s="6"/>
-      <c r="I43" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="J43" s="15">
+      <c r="I43" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="J43" s="11">
         <v>1</v>
       </c>
       <c r="K43" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L43" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M43" s="17">
+      <c r="L43" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M43" s="13">
         <v>0.47</v>
       </c>
-      <c r="N43" s="18">
+      <c r="N43" s="14">
         <f t="shared" si="4"/>
         <v>0.47</v>
       </c>
-      <c r="O43" s="17">
+      <c r="O43" s="13">
         <v>0.47</v>
       </c>
-      <c r="P43" s="18">
+      <c r="P43" s="14">
         <f t="shared" si="2"/>
         <v>2.3499999999999996</v>
       </c>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A44" s="12">
+      <c r="A44" s="9">
         <f t="shared" si="3"/>
         <v>42</v>
       </c>
-      <c r="B44" s="13"/>
-      <c r="C44" s="14" t="s">
+      <c r="B44" s="35"/>
+      <c r="C44" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="E44" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="D44" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="E44" s="14" t="s">
-        <v>187</v>
-      </c>
-      <c r="F44" s="14" t="s">
-        <v>184</v>
+      <c r="F44" s="10" t="s">
+        <v>182</v>
       </c>
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
-      <c r="I44" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="J44" s="15">
+      <c r="I44" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="J44" s="11">
         <v>1</v>
       </c>
       <c r="K44" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L44" s="16" t="s">
-        <v>238</v>
-      </c>
-      <c r="M44" s="17">
+      <c r="L44" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="M44" s="13">
         <v>0.19600000000000001</v>
       </c>
-      <c r="N44" s="18">
+      <c r="N44" s="14">
         <f t="shared" si="4"/>
         <v>0.19600000000000001</v>
       </c>
-      <c r="O44" s="17">
+      <c r="O44" s="13">
         <v>1.96</v>
       </c>
-      <c r="P44" s="18">
+      <c r="P44" s="14">
         <v>1.96</v>
       </c>
       <c r="Q44" s="6" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="45" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A45" s="12">
+      <c r="A45" s="9">
         <f t="shared" si="3"/>
         <v>43</v>
       </c>
-      <c r="B45" s="13"/>
-      <c r="C45" s="14" t="s">
+      <c r="B45" s="35"/>
+      <c r="C45" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="E45" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="D45" s="14" t="s">
-        <v>190</v>
-      </c>
-      <c r="E45" s="14" t="s">
-        <v>191</v>
-      </c>
-      <c r="F45" s="14" t="s">
-        <v>188</v>
+      <c r="F45" s="10" t="s">
+        <v>186</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="H45" s="6"/>
-      <c r="I45" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="J45" s="15">
+      <c r="I45" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="J45" s="11">
         <v>1</v>
       </c>
       <c r="K45" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L45" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M45" s="17">
+      <c r="L45" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M45" s="13">
         <v>0.44800000000000001</v>
       </c>
-      <c r="N45" s="18">
+      <c r="N45" s="14">
         <f t="shared" si="4"/>
         <v>0.44800000000000001</v>
       </c>
-      <c r="O45" s="17">
+      <c r="O45" s="13">
         <v>2.21</v>
       </c>
-      <c r="P45" s="18">
+      <c r="P45" s="14">
         <f t="shared" si="2"/>
         <v>11.05</v>
       </c>
       <c r="Q45" s="6" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A46" s="12">
+      <c r="A46" s="9">
         <f t="shared" si="3"/>
         <v>44</v>
       </c>
-      <c r="B46" s="13"/>
-      <c r="C46" s="14" t="s">
+      <c r="B46" s="35"/>
+      <c r="C46" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="E46" s="10" t="s">
         <v>193</v>
       </c>
-      <c r="D46" s="14" t="s">
-        <v>194</v>
-      </c>
-      <c r="E46" s="14" t="s">
-        <v>195</v>
-      </c>
-      <c r="F46" s="14" t="s">
-        <v>192</v>
+      <c r="F46" s="10" t="s">
+        <v>190</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="H46" s="6"/>
-      <c r="I46" s="14" t="s">
-        <v>192</v>
-      </c>
-      <c r="J46" s="15">
+      <c r="I46" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="J46" s="11">
         <v>1</v>
       </c>
       <c r="K46" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L46" s="16" t="s">
-        <v>240</v>
-      </c>
-      <c r="M46" s="17">
+      <c r="L46" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="M46" s="13">
         <v>0.52900000000000003</v>
       </c>
-      <c r="N46" s="18">
+      <c r="N46" s="14">
         <f t="shared" si="4"/>
         <v>0.52900000000000003</v>
       </c>
-      <c r="O46" s="17">
+      <c r="O46" s="13">
         <v>0.52900000000000003</v>
       </c>
-      <c r="P46" s="18">
+      <c r="P46" s="14">
         <f t="shared" si="2"/>
         <v>2.645</v>
       </c>
       <c r="Q46" s="6"/>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A47" s="12">
+      <c r="A47" s="9">
         <f t="shared" si="3"/>
         <v>45</v>
       </c>
-      <c r="B47" s="13"/>
-      <c r="C47" s="14" t="s">
+      <c r="B47" s="35"/>
+      <c r="C47" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="E47" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="D47" s="14" t="s">
-        <v>198</v>
-      </c>
-      <c r="E47" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="F47" s="14" t="s">
-        <v>196</v>
+      <c r="F47" s="10" t="s">
+        <v>194</v>
       </c>
       <c r="G47" s="6" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="H47" s="6"/>
-      <c r="I47" s="14" t="s">
-        <v>196</v>
-      </c>
-      <c r="J47" s="15">
+      <c r="I47" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="J47" s="11">
         <v>1</v>
       </c>
       <c r="K47" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L47" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M47" s="17">
+      <c r="L47" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M47" s="13">
         <v>0.51</v>
       </c>
-      <c r="N47" s="18">
+      <c r="N47" s="14">
         <f t="shared" si="4"/>
         <v>0.51</v>
       </c>
-      <c r="O47" s="17">
+      <c r="O47" s="13">
         <v>0.51</v>
       </c>
-      <c r="P47" s="18">
+      <c r="P47" s="14">
         <f t="shared" si="2"/>
         <v>2.5499999999999998</v>
       </c>
       <c r="Q47" s="6"/>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A48" s="12">
+      <c r="A48" s="9">
         <f t="shared" si="3"/>
         <v>46</v>
       </c>
-      <c r="B48" s="13"/>
-      <c r="C48" s="14" t="s">
+      <c r="B48" s="35"/>
+      <c r="C48" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="E48" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="D48" s="14" t="s">
-        <v>202</v>
-      </c>
-      <c r="E48" s="14" t="s">
-        <v>203</v>
-      </c>
-      <c r="F48" s="14" t="s">
-        <v>200</v>
+      <c r="F48" s="10" t="s">
+        <v>198</v>
       </c>
       <c r="G48" s="6"/>
       <c r="H48" s="6"/>
-      <c r="I48" s="14" t="s">
-        <v>200</v>
-      </c>
-      <c r="J48" s="15">
+      <c r="I48" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="J48" s="11">
         <v>1</v>
       </c>
       <c r="K48" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L48" s="16" t="s">
-        <v>238</v>
-      </c>
-      <c r="M48" s="17">
+      <c r="L48" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="M48" s="13">
         <v>7.92</v>
       </c>
-      <c r="N48" s="18">
+      <c r="N48" s="14">
         <f t="shared" si="4"/>
         <v>7.92</v>
       </c>
-      <c r="O48" s="17">
+      <c r="O48" s="13">
         <v>39.6</v>
       </c>
-      <c r="P48" s="18">
+      <c r="P48" s="14">
         <v>39.6</v>
       </c>
       <c r="Q48" s="6"/>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A49" s="12">
+      <c r="A49" s="9">
         <f t="shared" si="3"/>
         <v>47</v>
       </c>
-      <c r="B49" s="13"/>
-      <c r="C49" s="14" t="s">
+      <c r="B49" s="36"/>
+      <c r="C49" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="D49" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="E49" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="D49" s="14" t="s">
-        <v>206</v>
-      </c>
-      <c r="E49" s="14" t="s">
-        <v>207</v>
-      </c>
-      <c r="F49" s="14" t="s">
-        <v>204</v>
+      <c r="F49" s="10" t="s">
+        <v>202</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="H49" s="6"/>
-      <c r="I49" s="14" t="s">
-        <v>204</v>
-      </c>
-      <c r="J49" s="15">
+      <c r="I49" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="J49" s="11">
         <v>1</v>
       </c>
       <c r="K49" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L49" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M49" s="17">
+      <c r="L49" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M49" s="13">
         <v>2.31</v>
       </c>
-      <c r="N49" s="18">
+      <c r="N49" s="14">
         <f t="shared" si="4"/>
         <v>2.31</v>
       </c>
-      <c r="O49" s="17">
+      <c r="O49" s="13">
         <v>2.31</v>
       </c>
-      <c r="P49" s="18">
+      <c r="P49" s="14">
         <f t="shared" si="2"/>
         <v>11.55</v>
       </c>
       <c r="Q49" s="6"/>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A50" s="12">
+      <c r="A50" s="9">
         <f t="shared" si="3"/>
         <v>48</v>
       </c>
-      <c r="B50" s="13" t="s">
-        <v>230</v>
-      </c>
-      <c r="C50" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="D50" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="E50" s="14" t="s">
+      <c r="B50" s="30" t="s">
+        <v>228</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D50" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="F50" s="14" t="s">
-        <v>76</v>
+      <c r="E50" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="F50" s="10" t="s">
+        <v>74</v>
       </c>
       <c r="G50" s="6"/>
       <c r="H50" s="6"/>
-      <c r="I50" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="J50" s="15">
+      <c r="I50" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J50" s="11">
         <v>1</v>
       </c>
       <c r="K50" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L50" s="16" t="s">
-        <v>238</v>
-      </c>
-      <c r="M50" s="17">
+      <c r="L50" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="M50" s="13">
         <v>0.48</v>
       </c>
-      <c r="N50" s="18">
+      <c r="N50" s="14">
         <f t="shared" si="4"/>
         <v>0.48</v>
       </c>
-      <c r="O50" s="17">
+      <c r="O50" s="13">
         <v>0.48</v>
       </c>
-      <c r="P50" s="18">
+      <c r="P50" s="14">
         <f t="shared" si="2"/>
         <v>2.4</v>
       </c>
       <c r="Q50" s="6"/>
     </row>
     <row r="51" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A51" s="12">
+      <c r="A51" s="9">
         <f t="shared" si="3"/>
         <v>49</v>
       </c>
-      <c r="B51" s="13"/>
-      <c r="C51" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="D51" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="E51" s="14" t="s">
+      <c r="B51" s="30"/>
+      <c r="C51" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="D51" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="F51" s="14" t="s">
-        <v>79</v>
+      <c r="E51" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F51" s="10" t="s">
+        <v>77</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H51" s="6"/>
-      <c r="I51" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="J51" s="15">
+      <c r="I51" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="J51" s="11">
         <v>2</v>
       </c>
       <c r="K51" s="6">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L51" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M51" s="17">
+      <c r="L51" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M51" s="13">
         <v>1.92</v>
       </c>
-      <c r="N51" s="18">
+      <c r="N51" s="14">
         <f t="shared" si="4"/>
         <v>3.84</v>
       </c>
-      <c r="O51" s="17">
+      <c r="O51" s="13">
         <v>1.744</v>
       </c>
-      <c r="P51" s="18">
+      <c r="P51" s="14">
         <f t="shared" si="2"/>
         <v>17.440000000000001</v>
       </c>
       <c r="Q51" s="6"/>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A52" s="12">
+      <c r="A52" s="9">
         <f t="shared" si="3"/>
         <v>50</v>
       </c>
-      <c r="B52" s="13"/>
-      <c r="C52" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="D52" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="E52" s="14" t="s">
+      <c r="B52" s="30"/>
+      <c r="C52" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="D52" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="F52" s="14" t="s">
-        <v>82</v>
+      <c r="E52" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F52" s="10" t="s">
+        <v>80</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="H52" s="6"/>
-      <c r="I52" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="J52" s="15">
+      <c r="I52" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="J52" s="11">
         <v>1</v>
       </c>
       <c r="K52" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L52" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M52" s="17">
+      <c r="L52" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M52" s="13">
         <v>1.29</v>
       </c>
-      <c r="N52" s="18">
+      <c r="N52" s="14">
         <f t="shared" si="4"/>
         <v>1.29</v>
       </c>
-      <c r="O52" s="17">
+      <c r="O52" s="13">
         <v>1.29</v>
       </c>
-      <c r="P52" s="18">
+      <c r="P52" s="14">
         <f t="shared" si="2"/>
         <v>6.45</v>
       </c>
       <c r="Q52" s="6" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="53" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A53" s="12">
+      <c r="A53" s="9">
         <f t="shared" si="3"/>
         <v>51</v>
       </c>
-      <c r="B53" s="13"/>
-      <c r="C53" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="D53" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="E53" s="14" t="s">
+      <c r="B53" s="30"/>
+      <c r="C53" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="D53" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="F53" s="14" t="s">
-        <v>85</v>
+      <c r="E53" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="F53" s="10" t="s">
+        <v>83</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H53" s="6"/>
-      <c r="I53" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="J53" s="15">
+      <c r="I53" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="J53" s="11">
         <v>1</v>
       </c>
       <c r="K53" s="6">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L53" s="16" t="s">
-        <v>238</v>
-      </c>
-      <c r="M53" s="17">
+      <c r="L53" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="M53" s="13">
         <v>0.4</v>
       </c>
-      <c r="N53" s="18">
+      <c r="N53" s="14">
         <f>M53*J53</f>
         <v>0.4</v>
       </c>
-      <c r="O53" s="17">
+      <c r="O53" s="13">
         <v>4</v>
       </c>
-      <c r="P53" s="18">
+      <c r="P53" s="14">
         <v>4</v>
       </c>
       <c r="Q53" s="6"/>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A54" s="12">
+      <c r="A54" s="9">
         <f t="shared" si="3"/>
         <v>52</v>
       </c>
-      <c r="B54" s="13"/>
-      <c r="C54" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="D54" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="E54" s="14" t="s">
+      <c r="B54" s="30"/>
+      <c r="C54" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D54" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="F54" s="14" t="s">
-        <v>98</v>
+      <c r="E54" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="F54" s="10" t="s">
+        <v>96</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="H54" s="6"/>
-      <c r="I54" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="J54" s="15">
+      <c r="I54" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="J54" s="11">
         <v>2</v>
       </c>
       <c r="K54" s="6">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L54" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M54" s="17">
+      <c r="L54" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M54" s="13">
         <v>1.5</v>
       </c>
-      <c r="N54" s="18">
+      <c r="N54" s="14">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="O54" s="17">
+      <c r="O54" s="13">
         <v>1.5</v>
       </c>
-      <c r="P54" s="18">
+      <c r="P54" s="14">
         <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="Q54" s="6"/>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A55" s="12">
+      <c r="A55" s="9">
         <f t="shared" si="3"/>
         <v>53</v>
       </c>
-      <c r="B55" s="13"/>
-      <c r="C55" s="14" t="s">
+      <c r="B55" s="30"/>
+      <c r="C55" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D55" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E55" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="D55" s="14" t="s">
+      <c r="F55" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="E55" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="F55" s="14" t="s">
-        <v>109</v>
-      </c>
       <c r="G55" s="6" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="H55" s="6"/>
-      <c r="I55" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="J55" s="15">
+      <c r="I55" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="J55" s="11">
         <v>2</v>
       </c>
       <c r="K55" s="6">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L55" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="M55" s="17">
+      <c r="L55" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="M55" s="13">
         <v>0.13</v>
       </c>
-      <c r="N55" s="18">
+      <c r="N55" s="14">
         <f>M55*J55</f>
         <v>0.26</v>
       </c>
-      <c r="O55" s="17">
+      <c r="O55" s="13">
         <v>0.106</v>
       </c>
-      <c r="P55" s="18">
+      <c r="P55" s="14">
         <f>O55*K55</f>
         <v>1.06</v>
       </c>
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A56" s="12">
+      <c r="A56" s="9">
         <f t="shared" si="3"/>
         <v>54</v>
       </c>
-      <c r="B56" s="13"/>
-      <c r="C56" s="22" t="s">
+      <c r="B56" s="30"/>
+      <c r="C56" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="D56" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="E56" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="D56" s="22" t="s">
-        <v>103</v>
-      </c>
-      <c r="E56" s="22" t="s">
-        <v>104</v>
-      </c>
-      <c r="F56" s="22" t="s">
-        <v>104</v>
-      </c>
-      <c r="G56" s="23"/>
-      <c r="H56" s="23"/>
-      <c r="I56" s="22" t="s">
-        <v>101</v>
-      </c>
-      <c r="J56" s="23">
+      <c r="F56" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="G56" s="19"/>
+      <c r="H56" s="19"/>
+      <c r="I56" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="J56" s="19">
         <v>4</v>
       </c>
-      <c r="K56" s="23">
+      <c r="K56" s="19">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L56" s="23" t="s">
-        <v>233</v>
-      </c>
-      <c r="M56" s="23"/>
-      <c r="N56" s="24">
+      <c r="L56" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="M56" s="19"/>
+      <c r="N56" s="20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O56" s="25"/>
-      <c r="P56" s="24">
+      <c r="O56" s="21"/>
+      <c r="P56" s="20">
         <f>O56*K56</f>
         <v>0</v>
       </c>
-      <c r="Q56" s="23"/>
+      <c r="Q56" s="19"/>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A57" s="20"/>
-      <c r="B57" s="20"/>
-      <c r="C57" s="22" t="s">
-        <v>172</v>
-      </c>
-      <c r="D57" s="22" t="s">
-        <v>173</v>
-      </c>
-      <c r="E57" s="22" t="s">
+      <c r="A57" s="16"/>
+      <c r="B57" s="16"/>
+      <c r="C57" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="D57" s="18" t="s">
         <v>171</v>
       </c>
-      <c r="F57" s="22" t="s">
-        <v>171</v>
-      </c>
-      <c r="G57" s="23"/>
-      <c r="H57" s="23"/>
-      <c r="I57" s="22" t="s">
-        <v>171</v>
-      </c>
-      <c r="J57" s="23">
+      <c r="E57" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="F57" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="G57" s="19"/>
+      <c r="H57" s="19"/>
+      <c r="I57" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="J57" s="19">
         <v>1</v>
       </c>
-      <c r="K57" s="23">
+      <c r="K57" s="19">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L57" s="23" t="s">
-        <v>233</v>
-      </c>
-      <c r="M57" s="23"/>
-      <c r="N57" s="24">
+      <c r="L57" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="M57" s="19"/>
+      <c r="N57" s="20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O57" s="25"/>
-      <c r="P57" s="24">
+      <c r="O57" s="21"/>
+      <c r="P57" s="20">
         <f>O57*K57</f>
         <v>0</v>
       </c>
-      <c r="Q57" s="23"/>
+      <c r="Q57" s="19"/>
     </row>
     <row r="58" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C58" s="20"/>
-      <c r="D58" s="20"/>
-      <c r="E58" s="20"/>
-      <c r="F58" s="20"/>
-      <c r="G58" s="20"/>
-      <c r="H58" s="20"/>
-      <c r="I58" s="20"/>
-      <c r="J58" s="20"/>
-      <c r="K58" s="30" t="s">
-        <v>291</v>
-      </c>
-      <c r="L58" s="30"/>
-      <c r="M58" s="31"/>
-      <c r="N58" s="32">
+      <c r="C58" s="16"/>
+      <c r="D58" s="16"/>
+      <c r="E58" s="16"/>
+      <c r="F58" s="16"/>
+      <c r="G58" s="16"/>
+      <c r="H58" s="16"/>
+      <c r="I58" s="16"/>
+      <c r="J58" s="16"/>
+      <c r="K58" s="26" t="s">
+        <v>289</v>
+      </c>
+      <c r="L58" s="26"/>
+      <c r="M58" s="27"/>
+      <c r="N58" s="28">
         <f>SUM(N3:N55)</f>
         <v>70.28900000000003</v>
       </c>
-      <c r="O58" s="30"/>
-      <c r="P58" s="33">
+      <c r="O58" s="26"/>
+      <c r="P58" s="29">
         <f>SUM(P3:P55)</f>
         <v>324.673</v>
       </c>
@@ -4467,13 +4513,13 @@
     <row r="59" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B42:B49"/>
     <mergeCell ref="B50:B56"/>
     <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="B3:B18"/>
-    <mergeCell ref="B19:B22"/>
-    <mergeCell ref="B26:B39"/>
-    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="B3:B19"/>
+    <mergeCell ref="B27:B40"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="B43:B49"/>
   </mergeCells>
   <conditionalFormatting sqref="N3:N57">
     <cfRule type="dataBar" priority="4">

</xml_diff>

<commit_message>
C15 and C20 changed to 0.1uF/100V (CC0603KRX7R0BB104). Schematic, lib, PCB and BOM updated.
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/SM_Top_PCB_DigiKey.xlsx
+++ b/Deliverables/SM_Top Board/_BOM/SM_Top_PCB_DigiKey.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20376"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Github\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{090EA106-0B90-46AE-AD17-93E34983BAEB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8CE3DF8-60A6-47CE-9AA5-5159F2445391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="297">
   <si>
     <t>Description</t>
   </si>
@@ -153,13 +153,7 @@
     <t>CL10A475KA8NQNC</t>
   </si>
   <si>
-    <t>CAP CER 10000PF 100V X7R 0603</t>
-  </si>
-  <si>
     <t>C15, C20</t>
-  </si>
-  <si>
-    <t>CL10B103KC8NNNC</t>
   </si>
   <si>
     <t>220nF</t>
@@ -933,10 +927,10 @@
     <t>-------</t>
   </si>
   <si>
-    <t>0.01uF</t>
-  </si>
-  <si>
-    <t>C0603C103K1RAC3190</t>
+    <t>CC0603KRX7R0BB104</t>
+  </si>
+  <si>
+    <t>CAP CER 0.1UF 100V X7R 0603</t>
   </si>
 </sst>
 </file>
@@ -2092,7 +2086,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="109" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B1" s="110"/>
       <c r="C1" s="110"/>
@@ -2118,10 +2112,10 @@
     </row>
     <row r="2" spans="1:22" s="82" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="75" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B2" s="76" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C2" s="77" t="s">
         <v>0</v>
@@ -2130,58 +2124,58 @@
         <v>1</v>
       </c>
       <c r="E2" s="76" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F2" s="77" t="s">
         <v>2</v>
       </c>
       <c r="G2" s="76" t="s">
+        <v>194</v>
+      </c>
+      <c r="H2" s="77" t="s">
+        <v>195</v>
+      </c>
+      <c r="I2" s="76" t="s">
         <v>196</v>
       </c>
-      <c r="H2" s="77" t="s">
+      <c r="J2" s="77" t="s">
         <v>197</v>
       </c>
-      <c r="I2" s="76" t="s">
+      <c r="K2" s="76" t="s">
         <v>198</v>
       </c>
-      <c r="J2" s="77" t="s">
+      <c r="L2" s="78" t="s">
+        <v>265</v>
+      </c>
+      <c r="M2" s="79" t="s">
+        <v>266</v>
+      </c>
+      <c r="N2" s="79" t="s">
         <v>199</v>
       </c>
-      <c r="K2" s="76" t="s">
+      <c r="O2" s="79" t="s">
         <v>200</v>
       </c>
-      <c r="L2" s="78" t="s">
-        <v>267</v>
-      </c>
-      <c r="M2" s="79" t="s">
-        <v>268</v>
-      </c>
-      <c r="N2" s="79" t="s">
+      <c r="P2" s="80" t="s">
         <v>201</v>
       </c>
-      <c r="O2" s="79" t="s">
+      <c r="Q2" s="79" t="s">
         <v>202</v>
       </c>
-      <c r="P2" s="80" t="s">
-        <v>203</v>
-      </c>
-      <c r="Q2" s="79" t="s">
-        <v>204</v>
-      </c>
       <c r="R2" s="80" t="s">
+        <v>260</v>
+      </c>
+      <c r="S2" s="79" t="s">
+        <v>261</v>
+      </c>
+      <c r="T2" s="80" t="s">
         <v>262</v>
       </c>
-      <c r="S2" s="79" t="s">
+      <c r="U2" s="79" t="s">
         <v>263</v>
       </c>
-      <c r="T2" s="80" t="s">
-        <v>264</v>
-      </c>
-      <c r="U2" s="79" t="s">
-        <v>265</v>
-      </c>
       <c r="V2" s="81" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="3" spans="1:22" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2189,25 +2183,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="106" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C3" s="95" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D3" s="61" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F3" s="22" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="22" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="I3" s="22" t="s">
         <v>3</v>
@@ -2256,7 +2250,7 @@
         <v>186.82000000000002</v>
       </c>
       <c r="V3" s="28" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" spans="1:22" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2265,7 +2259,7 @@
       </c>
       <c r="B4" s="107"/>
       <c r="C4" s="96" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D4" s="57" t="s">
         <v>7</v>
@@ -2277,10 +2271,10 @@
         <v>9</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>6</v>
@@ -2348,10 +2342,10 @@
         <v>14</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>10</v>
@@ -2407,22 +2401,22 @@
       </c>
       <c r="B6" s="107"/>
       <c r="C6" s="96" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D6" s="57" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>17</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>15</v>
@@ -2471,7 +2465,7 @@
         <v>195.72</v>
       </c>
       <c r="V6" s="29" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2480,22 +2474,22 @@
       </c>
       <c r="B7" s="107"/>
       <c r="C7" s="96" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D7" s="57" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>20</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>18</v>
@@ -2544,7 +2538,7 @@
         <v>35.43</v>
       </c>
       <c r="V7" s="29" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2565,10 +2559,10 @@
         <v>24</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>21</v>
@@ -2636,10 +2630,10 @@
         <v>29</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>25</v>
@@ -2695,7 +2689,7 @@
       </c>
       <c r="B10" s="107"/>
       <c r="C10" s="96" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D10" s="57" t="s">
         <v>31</v>
@@ -2707,10 +2701,10 @@
         <v>32</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I10" s="6" t="s">
         <v>30</v>
@@ -2759,7 +2753,7 @@
         <v>56.15</v>
       </c>
       <c r="V10" s="29" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="11" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2768,7 +2762,7 @@
       </c>
       <c r="B11" s="107"/>
       <c r="C11" s="96" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D11" s="57" t="s">
         <v>33</v>
@@ -2780,10 +2774,10 @@
         <v>34</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I11" s="6" t="s">
         <v>10</v>
@@ -2839,7 +2833,7 @@
       </c>
       <c r="B12" s="107"/>
       <c r="C12" s="96" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D12" s="57" t="s">
         <v>36</v>
@@ -2851,10 +2845,10 @@
         <v>37</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="I12" s="6" t="s">
         <v>35</v>
@@ -2922,10 +2916,10 @@
         <v>41</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="I13" s="6" t="s">
         <v>38</v>
@@ -2981,25 +2975,25 @@
       </c>
       <c r="B14" s="107"/>
       <c r="C14" s="97" t="s">
+        <v>296</v>
+      </c>
+      <c r="D14" s="57" t="s">
         <v>42</v>
-      </c>
-      <c r="D14" s="57" t="s">
-        <v>43</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>28</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>44</v>
+        <v>295</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="H14" s="17" t="s">
-        <v>298</v>
+        <v>214</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>269</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>297</v>
+        <v>6</v>
       </c>
       <c r="J14" s="7">
         <v>2</v>
@@ -3052,25 +3046,25 @@
       </c>
       <c r="B15" s="107"/>
       <c r="C15" s="97" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D15" s="58" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="J15" s="7">
         <v>4</v>
@@ -3123,25 +3117,25 @@
       </c>
       <c r="B16" s="107"/>
       <c r="C16" s="96" t="s">
+        <v>250</v>
+      </c>
+      <c r="D16" s="59" t="s">
+        <v>251</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D16" s="59" t="s">
+      <c r="F16" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>255</v>
-      </c>
       <c r="G16" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="J16" s="3">
         <v>4</v>
@@ -3194,25 +3188,25 @@
       </c>
       <c r="B17" s="107"/>
       <c r="C17" s="96" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D17" s="57" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>28</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -3268,7 +3262,7 @@
         <v>26</v>
       </c>
       <c r="D18" s="57" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>28</v>
@@ -3277,13 +3271,13 @@
         <v>29</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="J18" s="7">
         <v>1</v>
@@ -3329,7 +3323,7 @@
         <v>6.9500000000000011</v>
       </c>
       <c r="V18" s="31" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="19" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3338,25 +3332,25 @@
       </c>
       <c r="B19" s="108"/>
       <c r="C19" s="98" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" s="60" t="s">
+        <v>51</v>
+      </c>
+      <c r="E19" s="32" t="s">
         <v>52</v>
       </c>
-      <c r="D19" s="60" t="s">
+      <c r="F19" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="E19" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="F19" s="32" t="s">
-        <v>55</v>
-      </c>
       <c r="G19" s="32" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="I19" s="32" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J19" s="35">
         <v>4</v>
@@ -3408,28 +3402,28 @@
         <v>18</v>
       </c>
       <c r="B20" s="106" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C20" s="95" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="D20" s="61" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E20" s="22" t="s">
+        <v>278</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="G20" s="22" t="s">
+        <v>225</v>
+      </c>
+      <c r="H20" s="48" t="s">
+        <v>239</v>
+      </c>
+      <c r="I20" s="22" t="s">
         <v>280</v>
-      </c>
-      <c r="F20" s="22" t="s">
-        <v>56</v>
-      </c>
-      <c r="G20" s="22" t="s">
-        <v>227</v>
-      </c>
-      <c r="H20" s="48" t="s">
-        <v>241</v>
-      </c>
-      <c r="I20" s="22" t="s">
-        <v>282</v>
       </c>
       <c r="J20" s="24">
         <v>1</v>
@@ -3475,7 +3469,7 @@
         <v>50.649999999999991</v>
       </c>
       <c r="V20" s="50" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="21" spans="1:22" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3484,25 +3478,25 @@
       </c>
       <c r="B21" s="107"/>
       <c r="C21" s="97" t="s">
+        <v>57</v>
+      </c>
+      <c r="D21" s="57" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="57" t="s">
-        <v>60</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>61</v>
-      </c>
       <c r="F21" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H21" s="17" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="J21" s="7">
         <v>8</v>
@@ -3548,7 +3542,7 @@
         <v>106.62400000000001</v>
       </c>
       <c r="V21" s="30" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="22" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3557,25 +3551,25 @@
       </c>
       <c r="B22" s="107"/>
       <c r="C22" s="97" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D22" s="57" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H22" s="17" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="J22" s="7">
         <v>1</v>
@@ -3628,25 +3622,25 @@
       </c>
       <c r="B23" s="108"/>
       <c r="C23" s="98" t="s">
+        <v>82</v>
+      </c>
+      <c r="D23" s="60" t="s">
+        <v>83</v>
+      </c>
+      <c r="E23" s="32" t="s">
         <v>84</v>
       </c>
-      <c r="D23" s="60" t="s">
-        <v>85</v>
-      </c>
-      <c r="E23" s="32" t="s">
-        <v>86</v>
-      </c>
       <c r="F23" s="32" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G23" s="32" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H23" s="32" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I23" s="32" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="J23" s="35">
         <v>1</v>
@@ -3698,28 +3692,28 @@
         <v>22</v>
       </c>
       <c r="B24" s="73" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C24" s="99" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D24" s="64" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E24" s="65" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F24" s="65" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G24" s="66" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H24" s="65" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I24" s="65" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="J24" s="67">
         <v>1</v>
@@ -3765,7 +3759,7 @@
         <v>22.14</v>
       </c>
       <c r="V24" s="71" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="25" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3773,28 +3767,28 @@
         <v>23</v>
       </c>
       <c r="B25" s="74" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C25" s="100" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D25" s="62" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E25" s="41" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F25" s="41" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G25" s="42" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="H25" s="41" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I25" s="41" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="J25" s="43">
         <v>1</v>
@@ -3846,28 +3840,28 @@
         <v>24</v>
       </c>
       <c r="B26" s="74" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C26" s="100" t="s">
+        <v>95</v>
+      </c>
+      <c r="D26" s="62" t="s">
+        <v>96</v>
+      </c>
+      <c r="E26" s="41" t="s">
         <v>97</v>
       </c>
-      <c r="D26" s="62" t="s">
-        <v>98</v>
-      </c>
-      <c r="E26" s="41" t="s">
-        <v>99</v>
-      </c>
       <c r="F26" s="41" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G26" s="42" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="H26" s="41" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I26" s="41" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="J26" s="43">
         <v>8</v>
@@ -3913,7 +3907,7 @@
         <v>898.30400000000009</v>
       </c>
       <c r="V26" s="47" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="27" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3921,28 +3915,28 @@
         <v>25</v>
       </c>
       <c r="B27" s="106" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C27" s="101" t="s">
+        <v>99</v>
+      </c>
+      <c r="D27" s="61" t="s">
+        <v>100</v>
+      </c>
+      <c r="E27" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="F27" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="D27" s="61" t="s">
-        <v>102</v>
-      </c>
-      <c r="E27" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="F27" s="22" t="s">
-        <v>103</v>
-      </c>
       <c r="G27" s="22" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H27" s="22" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I27" s="22" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="J27" s="24">
         <v>2</v>
@@ -3988,7 +3982,7 @@
         <v>1.6</v>
       </c>
       <c r="V27" s="55" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="28" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3997,25 +3991,25 @@
       </c>
       <c r="B28" s="107"/>
       <c r="C28" s="97" t="s">
+        <v>103</v>
+      </c>
+      <c r="D28" s="57" t="s">
+        <v>104</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F28" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="D28" s="57" t="s">
-        <v>106</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>107</v>
-      </c>
       <c r="G28" s="6" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H28" s="20" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J28" s="7">
         <v>2</v>
@@ -4068,25 +4062,25 @@
       </c>
       <c r="B29" s="107"/>
       <c r="C29" s="97" t="s">
+        <v>107</v>
+      </c>
+      <c r="D29" s="57" t="s">
+        <v>108</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F29" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="D29" s="57" t="s">
-        <v>110</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>111</v>
-      </c>
       <c r="G29" s="6" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H29" s="20" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -4132,7 +4126,7 @@
         <v>0.97</v>
       </c>
       <c r="V29" s="31" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="30" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4141,25 +4135,25 @@
       </c>
       <c r="B30" s="107"/>
       <c r="C30" s="96" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D30" s="57" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H30" s="20" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="J30" s="7">
         <v>1</v>
@@ -4212,25 +4206,25 @@
       </c>
       <c r="B31" s="107"/>
       <c r="C31" s="97" t="s">
+        <v>114</v>
+      </c>
+      <c r="D31" s="57" t="s">
+        <v>115</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F31" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="D31" s="57" t="s">
-        <v>117</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>118</v>
-      </c>
       <c r="G31" s="6" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H31" s="20" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J31" s="7">
         <v>4</v>
@@ -4283,25 +4277,25 @@
       </c>
       <c r="B32" s="107"/>
       <c r="C32" s="96" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D32" s="57" t="s">
+        <v>118</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F32" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="E32" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>122</v>
-      </c>
       <c r="G32" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="J32" s="7">
         <v>4</v>
@@ -4354,25 +4348,25 @@
       </c>
       <c r="B33" s="107"/>
       <c r="C33" s="97" t="s">
+        <v>122</v>
+      </c>
+      <c r="D33" s="57" t="s">
+        <v>123</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F33" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="D33" s="57" t="s">
-        <v>125</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>126</v>
-      </c>
       <c r="G33" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H33" s="53" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="J33" s="7">
         <v>8</v>
@@ -4425,25 +4419,25 @@
       </c>
       <c r="B34" s="107"/>
       <c r="C34" s="97" t="s">
+        <v>126</v>
+      </c>
+      <c r="D34" s="57" t="s">
+        <v>127</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F34" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="D34" s="57" t="s">
-        <v>129</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>130</v>
-      </c>
       <c r="G34" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="H34" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="H34" s="5" t="s">
-        <v>218</v>
-      </c>
       <c r="I34" s="6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J34" s="7">
         <v>1</v>
@@ -4496,25 +4490,25 @@
       </c>
       <c r="B35" s="107"/>
       <c r="C35" s="97" t="s">
+        <v>130</v>
+      </c>
+      <c r="D35" s="57" t="s">
+        <v>131</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F35" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="D35" s="57" t="s">
-        <v>133</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>134</v>
-      </c>
       <c r="G35" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H35" s="53" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -4567,25 +4561,25 @@
       </c>
       <c r="B36" s="107"/>
       <c r="C36" s="97" t="s">
+        <v>134</v>
+      </c>
+      <c r="D36" s="57" t="s">
+        <v>135</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F36" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="D36" s="57" t="s">
-        <v>137</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>138</v>
-      </c>
       <c r="G36" s="5" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="H36" s="53" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J36" s="7">
         <v>1</v>
@@ -4638,25 +4632,25 @@
       </c>
       <c r="B37" s="107"/>
       <c r="C37" s="97" t="s">
+        <v>138</v>
+      </c>
+      <c r="D37" s="57" t="s">
+        <v>139</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F37" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="D37" s="57" t="s">
-        <v>141</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>142</v>
-      </c>
       <c r="G37" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H37" s="53" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
@@ -4709,25 +4703,25 @@
       </c>
       <c r="B38" s="107"/>
       <c r="C38" s="97" t="s">
+        <v>142</v>
+      </c>
+      <c r="D38" s="57" t="s">
+        <v>143</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F38" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="D38" s="57" t="s">
-        <v>145</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F38" s="6" t="s">
-        <v>146</v>
-      </c>
       <c r="G38" s="5" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="H38" s="53" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J38" s="7">
         <v>1</v>
@@ -4780,25 +4774,25 @@
       </c>
       <c r="B39" s="107"/>
       <c r="C39" s="97" t="s">
+        <v>146</v>
+      </c>
+      <c r="D39" s="57" t="s">
+        <v>147</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F39" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="D39" s="57" t="s">
-        <v>149</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F39" s="6" t="s">
-        <v>150</v>
-      </c>
       <c r="G39" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>
@@ -4851,25 +4845,25 @@
       </c>
       <c r="B40" s="108"/>
       <c r="C40" s="98" t="s">
+        <v>150</v>
+      </c>
+      <c r="D40" s="60" t="s">
+        <v>151</v>
+      </c>
+      <c r="E40" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="F40" s="32" t="s">
         <v>152</v>
       </c>
-      <c r="D40" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="E40" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="F40" s="32" t="s">
-        <v>154</v>
-      </c>
       <c r="G40" s="36" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H40" s="54" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I40" s="32" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J40" s="35">
         <v>1</v>
@@ -4921,28 +4915,28 @@
         <v>39</v>
       </c>
       <c r="B41" s="106" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C41" s="101" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D41" s="61" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E41" s="22" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F41" s="22" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G41" s="83" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="H41" s="83" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I41" s="22" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J41" s="24">
         <v>1</v>
@@ -4987,7 +4981,7 @@
         <v>180</v>
       </c>
       <c r="V41" s="28" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="42" spans="1:22" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4996,25 +4990,25 @@
       </c>
       <c r="B42" s="108"/>
       <c r="C42" s="98" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D42" s="60" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E42" s="32" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F42" s="32" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G42" s="54" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="H42" s="84" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I42" s="32" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J42" s="35">
         <v>2</v>
@@ -5062,28 +5056,28 @@
         <v>41</v>
       </c>
       <c r="B43" s="106" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C43" s="101" t="s">
+        <v>163</v>
+      </c>
+      <c r="D43" s="61" t="s">
+        <v>164</v>
+      </c>
+      <c r="E43" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="D43" s="61" t="s">
-        <v>166</v>
-      </c>
-      <c r="E43" s="22" t="s">
-        <v>167</v>
-      </c>
       <c r="F43" s="22" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G43" s="85" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="H43" s="83" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I43" s="22" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J43" s="24">
         <v>1</v>
@@ -5129,7 +5123,7 @@
         <v>26.119999999999997</v>
       </c>
       <c r="V43" s="87" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="44" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5138,25 +5132,25 @@
       </c>
       <c r="B44" s="107"/>
       <c r="C44" s="97" t="s">
+        <v>167</v>
+      </c>
+      <c r="D44" s="57" t="s">
+        <v>168</v>
+      </c>
+      <c r="E44" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="D44" s="57" t="s">
-        <v>170</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>171</v>
-      </c>
       <c r="F44" s="6" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="H44" s="56" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J44" s="7">
         <v>1</v>
@@ -5209,25 +5203,25 @@
       </c>
       <c r="B45" s="107"/>
       <c r="C45" s="97" t="s">
+        <v>171</v>
+      </c>
+      <c r="D45" s="57" t="s">
+        <v>172</v>
+      </c>
+      <c r="E45" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="D45" s="57" t="s">
-        <v>174</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>175</v>
-      </c>
       <c r="F45" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="H45" s="56" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J45" s="7">
         <v>1</v>
@@ -5280,25 +5274,25 @@
       </c>
       <c r="B46" s="107"/>
       <c r="C46" s="97" t="s">
+        <v>175</v>
+      </c>
+      <c r="D46" s="57" t="s">
+        <v>176</v>
+      </c>
+      <c r="E46" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="D46" s="57" t="s">
-        <v>178</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>179</v>
-      </c>
       <c r="F46" s="6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H46" s="56" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J46" s="7">
         <v>1</v>
@@ -5351,25 +5345,25 @@
       </c>
       <c r="B47" s="107"/>
       <c r="C47" s="97" t="s">
+        <v>179</v>
+      </c>
+      <c r="D47" s="57" t="s">
+        <v>180</v>
+      </c>
+      <c r="E47" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="D47" s="57" t="s">
-        <v>182</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>183</v>
-      </c>
       <c r="F47" s="6" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="H47" s="56" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J47" s="7">
         <v>1</v>
@@ -5422,23 +5416,23 @@
       </c>
       <c r="B48" s="107"/>
       <c r="C48" s="97" t="s">
+        <v>183</v>
+      </c>
+      <c r="D48" s="57" t="s">
+        <v>184</v>
+      </c>
+      <c r="E48" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="D48" s="57" t="s">
-        <v>186</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>187</v>
-      </c>
       <c r="F48" s="6" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G48" s="5"/>
       <c r="H48" s="56" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J48" s="7">
         <v>1</v>
@@ -5491,25 +5485,25 @@
       </c>
       <c r="B49" s="108"/>
       <c r="C49" s="98" t="s">
+        <v>187</v>
+      </c>
+      <c r="D49" s="60" t="s">
+        <v>188</v>
+      </c>
+      <c r="E49" s="32" t="s">
         <v>189</v>
       </c>
-      <c r="D49" s="60" t="s">
-        <v>190</v>
-      </c>
-      <c r="E49" s="32" t="s">
-        <v>191</v>
-      </c>
       <c r="F49" s="32" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="G49" s="36" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="H49" s="84" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I49" s="32" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J49" s="35">
         <v>1</v>
@@ -5561,28 +5555,28 @@
         <v>48</v>
       </c>
       <c r="B50" s="106" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C50" s="101" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D50" s="22" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F50" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G50" s="25" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="H50" s="83" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I50" s="22" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J50" s="24">
         <v>1</v>
@@ -5635,25 +5629,25 @@
       </c>
       <c r="B51" s="107"/>
       <c r="C51" s="97" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="H51" s="56" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J51" s="7">
         <v>2</v>
@@ -5706,25 +5700,25 @@
       </c>
       <c r="B52" s="107"/>
       <c r="C52" s="97" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H52" s="56" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J52" s="7">
         <v>1</v>
@@ -5777,25 +5771,25 @@
       </c>
       <c r="B53" s="107"/>
       <c r="C53" s="97" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H53" s="56" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J53" s="7">
         <v>1</v>
@@ -5848,25 +5842,25 @@
       </c>
       <c r="B54" s="107"/>
       <c r="C54" s="97" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="H54" s="56" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J54" s="7">
         <v>2</v>
@@ -5919,25 +5913,25 @@
       </c>
       <c r="B55" s="107"/>
       <c r="C55" s="97" t="s">
+        <v>91</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E55" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="D55" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>95</v>
       </c>
       <c r="F55" s="6">
         <v>61300211121</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="H55" s="56" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J55" s="7">
         <v>2</v>
@@ -5990,21 +5984,21 @@
       </c>
       <c r="B56" s="107"/>
       <c r="C56" s="102" t="s">
+        <v>88</v>
+      </c>
+      <c r="D56" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E56" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D56" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="E56" s="11" t="s">
-        <v>92</v>
-      </c>
       <c r="F56" s="11" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G56" s="12"/>
       <c r="H56" s="12"/>
       <c r="I56" s="18" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J56" s="12">
         <v>4</v>
@@ -6042,7 +6036,7 @@
         <v>0</v>
       </c>
       <c r="V56" s="89" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="57" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6051,21 +6045,21 @@
       </c>
       <c r="B57" s="108"/>
       <c r="C57" s="103" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D57" s="90" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E57" s="90" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F57" s="90" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G57" s="91"/>
       <c r="H57" s="91"/>
       <c r="I57" s="33" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J57" s="91">
         <v>1</v>
@@ -6103,7 +6097,7 @@
         <v>0</v>
       </c>
       <c r="V57" s="94" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="58" spans="1:22" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -6115,7 +6109,7 @@
       <c r="H58" s="10"/>
       <c r="I58" s="10"/>
       <c r="J58" s="104" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="K58" s="104"/>
       <c r="L58" s="104"/>
@@ -6139,7 +6133,7 @@
     </row>
     <row r="59" spans="1:22" ht="18.75" x14ac:dyDescent="0.3">
       <c r="J59" s="105" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="K59" s="105"/>
       <c r="L59" s="105"/>

</xml_diff>

<commit_message>
Connector J4 changed in BOM as listed in issue #14
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/SM_Top_PCB_DigiKey.xlsx
+++ b/Deliverables/SM_Top Board/_BOM/SM_Top_PCB_DigiKey.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24228"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Temporary\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8CE3DF8-60A6-47CE-9AA5-5159F2445391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
   </bookViews>
   <sheets>
     <sheet name="SM_Top_PCB" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="297">
   <si>
     <t>Description</t>
   </si>
@@ -241,12 +240,6 @@
   </si>
   <si>
     <t>J3</t>
-  </si>
-  <si>
-    <t>B4P-VH-FB-B(LF)(SN)</t>
-  </si>
-  <si>
-    <t>CONN HEADER VERT 4POS 3.96MM</t>
   </si>
   <si>
     <t>J4</t>
@@ -931,12 +924,18 @@
   </si>
   <si>
     <t>CAP CER 0.1UF 100V X7R 0603</t>
+  </si>
+  <si>
+    <t>CONN HEADER VERT 4POS 2.5MM</t>
+  </si>
+  <si>
+    <t>B4B-XH-A(LF)(SN)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -1450,7 +1449,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1777,6 +1776,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2058,7 +2060,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:V59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2086,7 +2088,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="109" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B1" s="110"/>
       <c r="C1" s="110"/>
@@ -2112,10 +2114,10 @@
     </row>
     <row r="2" spans="1:22" s="82" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="75" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B2" s="76" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C2" s="77" t="s">
         <v>0</v>
@@ -2124,58 +2126,58 @@
         <v>1</v>
       </c>
       <c r="E2" s="76" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F2" s="77" t="s">
         <v>2</v>
       </c>
       <c r="G2" s="76" t="s">
+        <v>192</v>
+      </c>
+      <c r="H2" s="77" t="s">
+        <v>193</v>
+      </c>
+      <c r="I2" s="76" t="s">
         <v>194</v>
       </c>
-      <c r="H2" s="77" t="s">
+      <c r="J2" s="77" t="s">
         <v>195</v>
       </c>
-      <c r="I2" s="76" t="s">
+      <c r="K2" s="76" t="s">
         <v>196</v>
       </c>
-      <c r="J2" s="77" t="s">
+      <c r="L2" s="78" t="s">
+        <v>263</v>
+      </c>
+      <c r="M2" s="79" t="s">
+        <v>264</v>
+      </c>
+      <c r="N2" s="79" t="s">
         <v>197</v>
       </c>
-      <c r="K2" s="76" t="s">
+      <c r="O2" s="79" t="s">
         <v>198</v>
       </c>
-      <c r="L2" s="78" t="s">
-        <v>265</v>
-      </c>
-      <c r="M2" s="79" t="s">
-        <v>266</v>
-      </c>
-      <c r="N2" s="79" t="s">
+      <c r="P2" s="80" t="s">
         <v>199</v>
       </c>
-      <c r="O2" s="79" t="s">
+      <c r="Q2" s="79" t="s">
         <v>200</v>
       </c>
-      <c r="P2" s="80" t="s">
-        <v>201</v>
-      </c>
-      <c r="Q2" s="79" t="s">
-        <v>202</v>
-      </c>
       <c r="R2" s="80" t="s">
+        <v>258</v>
+      </c>
+      <c r="S2" s="79" t="s">
+        <v>259</v>
+      </c>
+      <c r="T2" s="80" t="s">
         <v>260</v>
       </c>
-      <c r="S2" s="79" t="s">
+      <c r="U2" s="79" t="s">
         <v>261</v>
       </c>
-      <c r="T2" s="80" t="s">
-        <v>262</v>
-      </c>
-      <c r="U2" s="79" t="s">
-        <v>263</v>
-      </c>
       <c r="V2" s="81" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="3" spans="1:22" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2183,25 +2185,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="106" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C3" s="95" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D3" s="61" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F3" s="22" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="22" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="I3" s="22" t="s">
         <v>3</v>
@@ -2250,7 +2252,7 @@
         <v>186.82000000000002</v>
       </c>
       <c r="V3" s="28" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4" spans="1:22" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2259,7 +2261,7 @@
       </c>
       <c r="B4" s="107"/>
       <c r="C4" s="96" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D4" s="57" t="s">
         <v>7</v>
@@ -2271,10 +2273,10 @@
         <v>9</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>6</v>
@@ -2342,10 +2344,10 @@
         <v>14</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>10</v>
@@ -2401,22 +2403,22 @@
       </c>
       <c r="B6" s="107"/>
       <c r="C6" s="96" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D6" s="57" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>17</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>15</v>
@@ -2465,7 +2467,7 @@
         <v>195.72</v>
       </c>
       <c r="V6" s="29" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="7" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2474,22 +2476,22 @@
       </c>
       <c r="B7" s="107"/>
       <c r="C7" s="96" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D7" s="57" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>20</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>18</v>
@@ -2538,7 +2540,7 @@
         <v>35.43</v>
       </c>
       <c r="V7" s="29" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2559,10 +2561,10 @@
         <v>24</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>21</v>
@@ -2630,10 +2632,10 @@
         <v>29</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>25</v>
@@ -2689,7 +2691,7 @@
       </c>
       <c r="B10" s="107"/>
       <c r="C10" s="96" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D10" s="57" t="s">
         <v>31</v>
@@ -2701,10 +2703,10 @@
         <v>32</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I10" s="6" t="s">
         <v>30</v>
@@ -2753,7 +2755,7 @@
         <v>56.15</v>
       </c>
       <c r="V10" s="29" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2762,7 +2764,7 @@
       </c>
       <c r="B11" s="107"/>
       <c r="C11" s="96" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D11" s="57" t="s">
         <v>33</v>
@@ -2774,10 +2776,10 @@
         <v>34</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I11" s="6" t="s">
         <v>10</v>
@@ -2833,7 +2835,7 @@
       </c>
       <c r="B12" s="107"/>
       <c r="C12" s="96" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D12" s="57" t="s">
         <v>36</v>
@@ -2845,10 +2847,10 @@
         <v>37</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="I12" s="6" t="s">
         <v>35</v>
@@ -2916,10 +2918,10 @@
         <v>41</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="I13" s="6" t="s">
         <v>38</v>
@@ -2975,7 +2977,7 @@
       </c>
       <c r="B14" s="107"/>
       <c r="C14" s="97" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D14" s="57" t="s">
         <v>42</v>
@@ -2984,13 +2986,13 @@
         <v>28</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I14" s="6" t="s">
         <v>6</v>
@@ -3046,22 +3048,22 @@
       </c>
       <c r="B15" s="107"/>
       <c r="C15" s="97" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="D15" s="58" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I15" s="6" t="s">
         <v>43</v>
@@ -3117,22 +3119,22 @@
       </c>
       <c r="B16" s="107"/>
       <c r="C16" s="96" t="s">
+        <v>248</v>
+      </c>
+      <c r="D16" s="59" t="s">
+        <v>249</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="D16" s="59" t="s">
+      <c r="F16" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>253</v>
-      </c>
       <c r="G16" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>43</v>
@@ -3188,7 +3190,7 @@
       </c>
       <c r="B17" s="107"/>
       <c r="C17" s="96" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D17" s="57" t="s">
         <v>45</v>
@@ -3200,10 +3202,10 @@
         <v>46</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I17" s="6" t="s">
         <v>44</v>
@@ -3271,10 +3273,10 @@
         <v>29</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I18" s="6" t="s">
         <v>47</v>
@@ -3323,7 +3325,7 @@
         <v>6.9500000000000011</v>
       </c>
       <c r="V18" s="31" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="19" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3344,10 +3346,10 @@
         <v>53</v>
       </c>
       <c r="G19" s="32" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="I19" s="32" t="s">
         <v>49</v>
@@ -3402,28 +3404,28 @@
         <v>18</v>
       </c>
       <c r="B20" s="106" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C20" s="95" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D20" s="61" t="s">
         <v>55</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="F20" s="22" t="s">
         <v>54</v>
       </c>
       <c r="G20" s="22" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H20" s="48" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="I20" s="22" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="J20" s="24">
         <v>1</v>
@@ -3469,7 +3471,7 @@
         <v>50.649999999999991</v>
       </c>
       <c r="V20" s="50" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="21" spans="1:22" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3490,13 +3492,13 @@
         <v>56</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H21" s="17" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="J21" s="7">
         <v>8</v>
@@ -3542,7 +3544,7 @@
         <v>106.62400000000001</v>
       </c>
       <c r="V21" s="30" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="22" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3551,25 +3553,25 @@
       </c>
       <c r="B22" s="107"/>
       <c r="C22" s="97" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D22" s="57" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H22" s="17" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="J22" s="7">
         <v>1</v>
@@ -3622,25 +3624,25 @@
       </c>
       <c r="B23" s="108"/>
       <c r="C23" s="98" t="s">
+        <v>80</v>
+      </c>
+      <c r="D23" s="60" t="s">
+        <v>81</v>
+      </c>
+      <c r="E23" s="32" t="s">
         <v>82</v>
       </c>
-      <c r="D23" s="60" t="s">
-        <v>83</v>
-      </c>
-      <c r="E23" s="32" t="s">
-        <v>84</v>
-      </c>
       <c r="F23" s="32" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G23" s="32" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H23" s="32" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I23" s="32" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="J23" s="35">
         <v>1</v>
@@ -3692,7 +3694,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="73" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C24" s="99" t="s">
         <v>61</v>
@@ -3701,19 +3703,19 @@
         <v>62</v>
       </c>
       <c r="E24" s="65" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F24" s="65" t="s">
         <v>60</v>
       </c>
       <c r="G24" s="66" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="H24" s="65" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I24" s="65" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="J24" s="67">
         <v>1</v>
@@ -3759,7 +3761,7 @@
         <v>22.14</v>
       </c>
       <c r="V24" s="71" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="25" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3767,28 +3769,28 @@
         <v>23</v>
       </c>
       <c r="B25" s="74" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C25" s="100" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D25" s="62" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E25" s="41" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F25" s="41" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G25" s="42" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="H25" s="41" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I25" s="41" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="J25" s="43">
         <v>1</v>
@@ -3840,28 +3842,28 @@
         <v>24</v>
       </c>
       <c r="B26" s="74" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C26" s="100" t="s">
+        <v>93</v>
+      </c>
+      <c r="D26" s="62" t="s">
+        <v>94</v>
+      </c>
+      <c r="E26" s="41" t="s">
         <v>95</v>
       </c>
-      <c r="D26" s="62" t="s">
-        <v>96</v>
-      </c>
-      <c r="E26" s="41" t="s">
-        <v>97</v>
-      </c>
       <c r="F26" s="41" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G26" s="42" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H26" s="41" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I26" s="41" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="J26" s="43">
         <v>8</v>
@@ -3907,7 +3909,7 @@
         <v>898.30400000000009</v>
       </c>
       <c r="V26" s="47" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="27" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3915,28 +3917,28 @@
         <v>25</v>
       </c>
       <c r="B27" s="106" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C27" s="101" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D27" s="61" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E27" s="22" t="s">
         <v>52</v>
       </c>
       <c r="F27" s="22" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G27" s="22" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H27" s="22" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I27" s="22" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J27" s="24">
         <v>2</v>
@@ -3982,7 +3984,7 @@
         <v>1.6</v>
       </c>
       <c r="V27" s="55" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="28" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3991,25 +3993,25 @@
       </c>
       <c r="B28" s="107"/>
       <c r="C28" s="97" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D28" s="57" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>52</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H28" s="20" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J28" s="7">
         <v>2</v>
@@ -4062,25 +4064,25 @@
       </c>
       <c r="B29" s="107"/>
       <c r="C29" s="97" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D29" s="57" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>52</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H29" s="20" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -4126,7 +4128,7 @@
         <v>0.97</v>
       </c>
       <c r="V29" s="31" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="30" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4135,25 +4137,25 @@
       </c>
       <c r="B30" s="107"/>
       <c r="C30" s="96" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="D30" s="57" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>52</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H30" s="20" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J30" s="7">
         <v>1</v>
@@ -4206,25 +4208,25 @@
       </c>
       <c r="B31" s="107"/>
       <c r="C31" s="97" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D31" s="57" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E31" s="6" t="s">
         <v>52</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H31" s="20" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="J31" s="7">
         <v>4</v>
@@ -4277,25 +4279,25 @@
       </c>
       <c r="B32" s="107"/>
       <c r="C32" s="96" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D32" s="57" t="s">
+        <v>116</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F32" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="E32" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>120</v>
-      </c>
       <c r="G32" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="J32" s="7">
         <v>4</v>
@@ -4348,25 +4350,25 @@
       </c>
       <c r="B33" s="107"/>
       <c r="C33" s="97" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D33" s="57" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>52</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H33" s="53" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J33" s="7">
         <v>8</v>
@@ -4419,25 +4421,25 @@
       </c>
       <c r="B34" s="107"/>
       <c r="C34" s="97" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D34" s="57" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>52</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G34" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="H34" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="H34" s="5" t="s">
-        <v>216</v>
-      </c>
       <c r="I34" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="J34" s="7">
         <v>1</v>
@@ -4490,25 +4492,25 @@
       </c>
       <c r="B35" s="107"/>
       <c r="C35" s="97" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D35" s="57" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>52</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H35" s="53" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -4561,25 +4563,25 @@
       </c>
       <c r="B36" s="107"/>
       <c r="C36" s="97" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D36" s="57" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>52</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="H36" s="53" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J36" s="7">
         <v>1</v>
@@ -4632,25 +4634,25 @@
       </c>
       <c r="B37" s="107"/>
       <c r="C37" s="97" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D37" s="57" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E37" s="6" t="s">
         <v>52</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H37" s="53" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
@@ -4703,25 +4705,25 @@
       </c>
       <c r="B38" s="107"/>
       <c r="C38" s="97" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D38" s="57" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>52</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="H38" s="53" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="J38" s="7">
         <v>1</v>
@@ -4774,25 +4776,25 @@
       </c>
       <c r="B39" s="107"/>
       <c r="C39" s="97" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D39" s="57" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>52</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>
@@ -4845,25 +4847,25 @@
       </c>
       <c r="B40" s="108"/>
       <c r="C40" s="98" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D40" s="60" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E40" s="32" t="s">
         <v>52</v>
       </c>
       <c r="F40" s="32" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G40" s="36" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H40" s="54" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I40" s="32" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J40" s="35">
         <v>1</v>
@@ -4915,28 +4917,28 @@
         <v>39</v>
       </c>
       <c r="B41" s="106" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C41" s="101" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D41" s="61" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E41" s="22" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F41" s="22" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="G41" s="83" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H41" s="83" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I41" s="22" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J41" s="24">
         <v>1</v>
@@ -4981,7 +4983,7 @@
         <v>180</v>
       </c>
       <c r="V41" s="28" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="42" spans="1:22" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4990,25 +4992,25 @@
       </c>
       <c r="B42" s="108"/>
       <c r="C42" s="98" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D42" s="60" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E42" s="32" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F42" s="32" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G42" s="54" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="H42" s="84" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I42" s="32" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J42" s="35">
         <v>2</v>
@@ -5056,28 +5058,28 @@
         <v>41</v>
       </c>
       <c r="B43" s="106" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C43" s="101" t="s">
+        <v>161</v>
+      </c>
+      <c r="D43" s="61" t="s">
+        <v>162</v>
+      </c>
+      <c r="E43" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="D43" s="61" t="s">
-        <v>164</v>
-      </c>
-      <c r="E43" s="22" t="s">
-        <v>165</v>
-      </c>
       <c r="F43" s="22" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="G43" s="85" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="H43" s="83" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I43" s="22" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J43" s="24">
         <v>1</v>
@@ -5123,7 +5125,7 @@
         <v>26.119999999999997</v>
       </c>
       <c r="V43" s="87" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="44" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5132,25 +5134,25 @@
       </c>
       <c r="B44" s="107"/>
       <c r="C44" s="97" t="s">
+        <v>165</v>
+      </c>
+      <c r="D44" s="57" t="s">
+        <v>166</v>
+      </c>
+      <c r="E44" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="D44" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>169</v>
-      </c>
       <c r="F44" s="6" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="H44" s="56" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J44" s="7">
         <v>1</v>
@@ -5203,25 +5205,25 @@
       </c>
       <c r="B45" s="107"/>
       <c r="C45" s="97" t="s">
+        <v>169</v>
+      </c>
+      <c r="D45" s="57" t="s">
+        <v>170</v>
+      </c>
+      <c r="E45" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="D45" s="57" t="s">
-        <v>172</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>173</v>
-      </c>
       <c r="F45" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="H45" s="56" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J45" s="7">
         <v>1</v>
@@ -5274,25 +5276,25 @@
       </c>
       <c r="B46" s="107"/>
       <c r="C46" s="97" t="s">
+        <v>173</v>
+      </c>
+      <c r="D46" s="57" t="s">
+        <v>174</v>
+      </c>
+      <c r="E46" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="D46" s="57" t="s">
-        <v>176</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>177</v>
-      </c>
       <c r="F46" s="6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="H46" s="56" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J46" s="7">
         <v>1</v>
@@ -5345,25 +5347,25 @@
       </c>
       <c r="B47" s="107"/>
       <c r="C47" s="97" t="s">
+        <v>177</v>
+      </c>
+      <c r="D47" s="57" t="s">
+        <v>178</v>
+      </c>
+      <c r="E47" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="D47" s="57" t="s">
-        <v>180</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>181</v>
-      </c>
       <c r="F47" s="6" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="H47" s="56" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J47" s="7">
         <v>1</v>
@@ -5416,23 +5418,23 @@
       </c>
       <c r="B48" s="107"/>
       <c r="C48" s="97" t="s">
+        <v>181</v>
+      </c>
+      <c r="D48" s="57" t="s">
+        <v>182</v>
+      </c>
+      <c r="E48" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="D48" s="57" t="s">
-        <v>184</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>185</v>
-      </c>
       <c r="F48" s="6" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G48" s="5"/>
       <c r="H48" s="56" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J48" s="7">
         <v>1</v>
@@ -5485,25 +5487,25 @@
       </c>
       <c r="B49" s="108"/>
       <c r="C49" s="98" t="s">
+        <v>185</v>
+      </c>
+      <c r="D49" s="60" t="s">
+        <v>186</v>
+      </c>
+      <c r="E49" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="D49" s="60" t="s">
-        <v>188</v>
-      </c>
-      <c r="E49" s="32" t="s">
-        <v>189</v>
-      </c>
       <c r="F49" s="32" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G49" s="36" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H49" s="84" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I49" s="32" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J49" s="35">
         <v>1</v>
@@ -5555,7 +5557,7 @@
         <v>48</v>
       </c>
       <c r="B50" s="106" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C50" s="101" t="s">
         <v>64</v>
@@ -5564,19 +5566,19 @@
         <v>65</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F50" s="22" t="s">
         <v>63</v>
       </c>
       <c r="G50" s="25" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="H50" s="83" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I50" s="22" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J50" s="24">
         <v>1</v>
@@ -5635,19 +5637,19 @@
         <v>68</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F51" s="6" t="s">
         <v>66</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="H51" s="56" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J51" s="7">
         <v>2</v>
@@ -5706,19 +5708,19 @@
         <v>71</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>69</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="H52" s="56" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J52" s="7">
         <v>1</v>
@@ -5770,71 +5772,65 @@
         <v>51</v>
       </c>
       <c r="B53" s="107"/>
-      <c r="C53" s="97" t="s">
-        <v>73</v>
-      </c>
-      <c r="D53" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="F53" s="6" t="s">
+      <c r="C53" s="102" t="s">
+        <v>295</v>
+      </c>
+      <c r="D53" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="G53" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="H53" s="56" t="s">
-        <v>269</v>
-      </c>
-      <c r="I53" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="J53" s="7">
+      <c r="E53" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="F53" s="11" t="s">
+        <v>296</v>
+      </c>
+      <c r="G53" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="H53" s="112" t="s">
+        <v>267</v>
+      </c>
+      <c r="I53" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="J53" s="12">
         <v>1</v>
       </c>
-      <c r="K53" s="5">
+      <c r="K53" s="12">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="L53" s="5">
+      <c r="L53" s="12">
         <f t="shared" si="5"/>
         <v>25</v>
       </c>
-      <c r="M53" s="5">
+      <c r="M53" s="12">
         <f t="shared" si="6"/>
         <v>100</v>
       </c>
-      <c r="N53" s="8">
-        <v>0.39</v>
-      </c>
-      <c r="O53" s="9">
+      <c r="N53" s="14"/>
+      <c r="O53" s="13">
         <f t="shared" si="7"/>
-        <v>0.39</v>
-      </c>
-      <c r="P53" s="8">
-        <v>0.39</v>
-      </c>
-      <c r="Q53" s="9">
+        <v>0</v>
+      </c>
+      <c r="P53" s="14"/>
+      <c r="Q53" s="13">
         <f t="shared" si="10"/>
-        <v>1.9500000000000002</v>
-      </c>
-      <c r="R53" s="9">
-        <v>0.372</v>
-      </c>
-      <c r="S53" s="9">
+        <v>0</v>
+      </c>
+      <c r="R53" s="13"/>
+      <c r="S53" s="13">
         <f t="shared" si="8"/>
-        <v>9.3000000000000007</v>
-      </c>
-      <c r="T53" s="9">
-        <v>0.2606</v>
-      </c>
-      <c r="U53" s="9">
+        <v>0</v>
+      </c>
+      <c r="T53" s="13"/>
+      <c r="U53" s="13">
         <f t="shared" si="9"/>
-        <v>26.06</v>
-      </c>
-      <c r="V53" s="29"/>
+        <v>0</v>
+      </c>
+      <c r="V53" s="89" t="s">
+        <v>288</v>
+      </c>
     </row>
     <row r="54" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="75">
@@ -5842,25 +5838,25 @@
       </c>
       <c r="B54" s="107"/>
       <c r="C54" s="97" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H54" s="56" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J54" s="7">
         <v>2</v>
@@ -5913,25 +5909,25 @@
       </c>
       <c r="B55" s="107"/>
       <c r="C55" s="97" t="s">
+        <v>89</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E55" s="6" t="s">
         <v>91</v>
-      </c>
-      <c r="D55" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>93</v>
       </c>
       <c r="F55" s="6">
         <v>61300211121</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H55" s="56" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J55" s="7">
         <v>2</v>
@@ -5984,21 +5980,21 @@
       </c>
       <c r="B56" s="107"/>
       <c r="C56" s="102" t="s">
+        <v>86</v>
+      </c>
+      <c r="D56" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E56" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="D56" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="E56" s="11" t="s">
-        <v>90</v>
-      </c>
       <c r="F56" s="11" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G56" s="12"/>
       <c r="H56" s="12"/>
       <c r="I56" s="18" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J56" s="12">
         <v>4</v>
@@ -6036,7 +6032,7 @@
         <v>0</v>
       </c>
       <c r="V56" s="89" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="57" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6045,21 +6041,21 @@
       </c>
       <c r="B57" s="108"/>
       <c r="C57" s="103" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D57" s="90" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E57" s="90" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F57" s="90" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G57" s="91"/>
       <c r="H57" s="91"/>
       <c r="I57" s="33" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J57" s="91">
         <v>1</v>
@@ -6097,7 +6093,7 @@
         <v>0</v>
       </c>
       <c r="V57" s="94" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="58" spans="1:22" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -6109,31 +6105,31 @@
       <c r="H58" s="10"/>
       <c r="I58" s="10"/>
       <c r="J58" s="104" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="K58" s="104"/>
       <c r="L58" s="104"/>
       <c r="M58" s="104"/>
       <c r="O58" s="21">
         <f>SUM(O3:O55)</f>
-        <v>69.440800000000024</v>
+        <v>69.050800000000024</v>
       </c>
       <c r="Q58" s="21">
         <f>SUM(Q3:Q55)</f>
-        <v>308.31899999999996</v>
+        <v>306.36899999999997</v>
       </c>
       <c r="S58" s="21">
         <f>SUM(S3:S57)</f>
-        <v>1267.0875000000003</v>
+        <v>1257.7875000000004</v>
       </c>
       <c r="U58" s="21">
         <f>SUM(U3:U57)</f>
-        <v>4284.1159999999991</v>
+        <v>4258.0559999999987</v>
       </c>
     </row>
     <row r="59" spans="1:22" ht="18.75" x14ac:dyDescent="0.3">
       <c r="J59" s="105" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="K59" s="105"/>
       <c r="L59" s="105"/>
@@ -6141,15 +6137,15 @@
       <c r="O59" s="63"/>
       <c r="Q59" s="63">
         <f>Q58/5</f>
-        <v>61.663799999999995</v>
+        <v>61.273799999999994</v>
       </c>
       <c r="S59" s="63">
         <f>S58/25</f>
-        <v>50.683500000000009</v>
+        <v>50.311500000000017</v>
       </c>
       <c r="U59" s="63">
         <f>U58/100</f>
-        <v>42.841159999999988</v>
+        <v>42.580559999999984</v>
       </c>
     </row>
   </sheetData>

</xml_diff>